<commit_message>
Decode Origin values in Auto MPG source dataset
Replace numeric Origin codes in sample_data/auto_mpg_data.xlsx with region labels (US/Europe/Asia) and align regression/model-construction QC logic and expectations with the new categorical values.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample_data/auto_mpg_data.xlsx
+++ b/sample_data/auto_mpg_data.xlsx
@@ -1488,8 +1488,8 @@
       <c r="G2">
         <v>70</v>
       </c>
-      <c r="H2">
-        <v>1</v>
+      <c r="H2" t="str">
+        <v>US</v>
       </c>
       <c r="I2" t="s">
         <v>0</v>
@@ -1525,8 +1525,8 @@
       <c r="G3">
         <v>70</v>
       </c>
-      <c r="H3">
-        <v>1</v>
+      <c r="H3" t="str">
+        <v>US</v>
       </c>
       <c r="I3" t="s">
         <v>1</v>
@@ -1562,8 +1562,8 @@
       <c r="G4">
         <v>70</v>
       </c>
-      <c r="H4">
-        <v>1</v>
+      <c r="H4" t="str">
+        <v>US</v>
       </c>
       <c r="I4" t="s">
         <v>2</v>
@@ -1599,8 +1599,8 @@
       <c r="G5">
         <v>70</v>
       </c>
-      <c r="H5">
-        <v>1</v>
+      <c r="H5" t="str">
+        <v>US</v>
       </c>
       <c r="I5" t="s">
         <v>3</v>
@@ -1636,8 +1636,8 @@
       <c r="G6">
         <v>70</v>
       </c>
-      <c r="H6">
-        <v>1</v>
+      <c r="H6" t="str">
+        <v>US</v>
       </c>
       <c r="I6" t="s">
         <v>4</v>
@@ -1673,8 +1673,8 @@
       <c r="G7">
         <v>70</v>
       </c>
-      <c r="H7">
-        <v>1</v>
+      <c r="H7" t="str">
+        <v>US</v>
       </c>
       <c r="I7" t="s">
         <v>5</v>
@@ -1710,8 +1710,8 @@
       <c r="G8">
         <v>70</v>
       </c>
-      <c r="H8">
-        <v>1</v>
+      <c r="H8" t="str">
+        <v>US</v>
       </c>
       <c r="I8" t="s">
         <v>6</v>
@@ -1747,8 +1747,8 @@
       <c r="G9">
         <v>70</v>
       </c>
-      <c r="H9">
-        <v>1</v>
+      <c r="H9" t="str">
+        <v>US</v>
       </c>
       <c r="I9" t="s">
         <v>7</v>
@@ -1784,8 +1784,8 @@
       <c r="G10">
         <v>70</v>
       </c>
-      <c r="H10">
-        <v>1</v>
+      <c r="H10" t="str">
+        <v>US</v>
       </c>
       <c r="I10" t="s">
         <v>8</v>
@@ -1821,8 +1821,8 @@
       <c r="G11">
         <v>70</v>
       </c>
-      <c r="H11">
-        <v>1</v>
+      <c r="H11" t="str">
+        <v>US</v>
       </c>
       <c r="I11" t="s">
         <v>9</v>
@@ -1858,8 +1858,8 @@
       <c r="G12">
         <v>70</v>
       </c>
-      <c r="H12">
-        <v>2</v>
+      <c r="H12" t="str">
+        <v>Europe</v>
       </c>
       <c r="I12" t="s">
         <v>10</v>
@@ -1895,8 +1895,8 @@
       <c r="G13">
         <v>70</v>
       </c>
-      <c r="H13">
-        <v>1</v>
+      <c r="H13" t="str">
+        <v>US</v>
       </c>
       <c r="I13" t="s">
         <v>11</v>
@@ -1932,8 +1932,8 @@
       <c r="G14">
         <v>70</v>
       </c>
-      <c r="H14">
-        <v>1</v>
+      <c r="H14" t="str">
+        <v>US</v>
       </c>
       <c r="I14" t="s">
         <v>12</v>
@@ -1969,8 +1969,8 @@
       <c r="G15">
         <v>70</v>
       </c>
-      <c r="H15">
-        <v>1</v>
+      <c r="H15" t="str">
+        <v>US</v>
       </c>
       <c r="I15" t="s">
         <v>13</v>
@@ -2006,8 +2006,8 @@
       <c r="G16">
         <v>70</v>
       </c>
-      <c r="H16">
-        <v>1</v>
+      <c r="H16" t="str">
+        <v>US</v>
       </c>
       <c r="I16" t="s">
         <v>14</v>
@@ -2043,8 +2043,8 @@
       <c r="G17">
         <v>70</v>
       </c>
-      <c r="H17">
-        <v>1</v>
+      <c r="H17" t="str">
+        <v>US</v>
       </c>
       <c r="I17" t="s">
         <v>15</v>
@@ -2080,8 +2080,8 @@
       <c r="G18">
         <v>70</v>
       </c>
-      <c r="H18">
-        <v>1</v>
+      <c r="H18" t="str">
+        <v>US</v>
       </c>
       <c r="I18" t="s">
         <v>16</v>
@@ -2117,8 +2117,8 @@
       <c r="G19">
         <v>70</v>
       </c>
-      <c r="H19">
-        <v>1</v>
+      <c r="H19" t="str">
+        <v>US</v>
       </c>
       <c r="I19" t="s">
         <v>17</v>
@@ -2154,8 +2154,8 @@
       <c r="G20">
         <v>70</v>
       </c>
-      <c r="H20">
-        <v>1</v>
+      <c r="H20" t="str">
+        <v>US</v>
       </c>
       <c r="I20" t="s">
         <v>18</v>
@@ -2191,8 +2191,8 @@
       <c r="G21">
         <v>70</v>
       </c>
-      <c r="H21">
-        <v>1</v>
+      <c r="H21" t="str">
+        <v>US</v>
       </c>
       <c r="I21" t="s">
         <v>19</v>
@@ -2228,8 +2228,8 @@
       <c r="G22">
         <v>70</v>
       </c>
-      <c r="H22">
-        <v>3</v>
+      <c r="H22" t="str">
+        <v>Asia</v>
       </c>
       <c r="I22" t="s">
         <v>20</v>
@@ -2265,8 +2265,8 @@
       <c r="G23">
         <v>70</v>
       </c>
-      <c r="H23">
-        <v>1</v>
+      <c r="H23" t="str">
+        <v>US</v>
       </c>
       <c r="I23" t="s">
         <v>21</v>
@@ -2302,8 +2302,8 @@
       <c r="G24">
         <v>70</v>
       </c>
-      <c r="H24">
-        <v>1</v>
+      <c r="H24" t="str">
+        <v>US</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
@@ -2339,8 +2339,8 @@
       <c r="G25">
         <v>70</v>
       </c>
-      <c r="H25">
-        <v>1</v>
+      <c r="H25" t="str">
+        <v>US</v>
       </c>
       <c r="I25" t="s">
         <v>23</v>
@@ -2376,8 +2376,8 @@
       <c r="G26">
         <v>70</v>
       </c>
-      <c r="H26">
-        <v>3</v>
+      <c r="H26" t="str">
+        <v>Asia</v>
       </c>
       <c r="I26" t="s">
         <v>24</v>
@@ -2413,8 +2413,8 @@
       <c r="G27">
         <v>70</v>
       </c>
-      <c r="H27">
-        <v>2</v>
+      <c r="H27" t="str">
+        <v>Europe</v>
       </c>
       <c r="I27" t="s">
         <v>25</v>
@@ -2450,8 +2450,8 @@
       <c r="G28">
         <v>70</v>
       </c>
-      <c r="H28">
-        <v>2</v>
+      <c r="H28" t="str">
+        <v>Europe</v>
       </c>
       <c r="I28" t="s">
         <v>26</v>
@@ -2487,8 +2487,8 @@
       <c r="G29">
         <v>70</v>
       </c>
-      <c r="H29">
-        <v>2</v>
+      <c r="H29" t="str">
+        <v>Europe</v>
       </c>
       <c r="I29" t="s">
         <v>27</v>
@@ -2524,8 +2524,8 @@
       <c r="G30">
         <v>70</v>
       </c>
-      <c r="H30">
-        <v>2</v>
+      <c r="H30" t="str">
+        <v>Europe</v>
       </c>
       <c r="I30" t="s">
         <v>28</v>
@@ -2561,8 +2561,8 @@
       <c r="G31">
         <v>70</v>
       </c>
-      <c r="H31">
-        <v>2</v>
+      <c r="H31" t="str">
+        <v>Europe</v>
       </c>
       <c r="I31" t="s">
         <v>29</v>
@@ -2598,8 +2598,8 @@
       <c r="G32">
         <v>70</v>
       </c>
-      <c r="H32">
-        <v>1</v>
+      <c r="H32" t="str">
+        <v>US</v>
       </c>
       <c r="I32" t="s">
         <v>30</v>
@@ -2635,8 +2635,8 @@
       <c r="G33">
         <v>70</v>
       </c>
-      <c r="H33">
-        <v>1</v>
+      <c r="H33" t="str">
+        <v>US</v>
       </c>
       <c r="I33" t="s">
         <v>31</v>
@@ -2672,8 +2672,8 @@
       <c r="G34">
         <v>70</v>
       </c>
-      <c r="H34">
-        <v>1</v>
+      <c r="H34" t="str">
+        <v>US</v>
       </c>
       <c r="I34" t="s">
         <v>32</v>
@@ -2709,8 +2709,8 @@
       <c r="G35">
         <v>70</v>
       </c>
-      <c r="H35">
-        <v>1</v>
+      <c r="H35" t="str">
+        <v>US</v>
       </c>
       <c r="I35" t="s">
         <v>33</v>
@@ -2746,8 +2746,8 @@
       <c r="G36">
         <v>70</v>
       </c>
-      <c r="H36">
-        <v>1</v>
+      <c r="H36" t="str">
+        <v>US</v>
       </c>
       <c r="I36" t="s">
         <v>34</v>
@@ -2783,8 +2783,8 @@
       <c r="G37">
         <v>71</v>
       </c>
-      <c r="H37">
-        <v>3</v>
+      <c r="H37" t="str">
+        <v>Asia</v>
       </c>
       <c r="I37" t="s">
         <v>24</v>
@@ -2820,8 +2820,8 @@
       <c r="G38">
         <v>71</v>
       </c>
-      <c r="H38">
-        <v>1</v>
+      <c r="H38" t="str">
+        <v>US</v>
       </c>
       <c r="I38" t="s">
         <v>35</v>
@@ -2857,8 +2857,8 @@
       <c r="G39">
         <v>71</v>
       </c>
-      <c r="H39">
-        <v>3</v>
+      <c r="H39" t="str">
+        <v>Asia</v>
       </c>
       <c r="I39" t="s">
         <v>36</v>
@@ -2894,8 +2894,8 @@
       <c r="G40">
         <v>71</v>
       </c>
-      <c r="H40">
-        <v>1</v>
+      <c r="H40" t="str">
+        <v>US</v>
       </c>
       <c r="I40" t="s">
         <v>37</v>
@@ -2931,8 +2931,8 @@
       <c r="G41">
         <v>71</v>
       </c>
-      <c r="H41">
-        <v>2</v>
+      <c r="H41" t="str">
+        <v>Europe</v>
       </c>
       <c r="I41" t="s">
         <v>38</v>
@@ -2968,8 +2968,8 @@
       <c r="G42">
         <v>71</v>
       </c>
-      <c r="H42">
-        <v>1</v>
+      <c r="H42" t="str">
+        <v>US</v>
       </c>
       <c r="I42" t="s">
         <v>30</v>
@@ -3005,8 +3005,8 @@
       <c r="G43">
         <v>71</v>
       </c>
-      <c r="H43">
-        <v>1</v>
+      <c r="H43" t="str">
+        <v>US</v>
       </c>
       <c r="I43" t="s">
         <v>39</v>
@@ -3042,8 +3042,8 @@
       <c r="G44">
         <v>71</v>
       </c>
-      <c r="H44">
-        <v>1</v>
+      <c r="H44" t="str">
+        <v>US</v>
       </c>
       <c r="I44" t="s">
         <v>0</v>
@@ -3079,8 +3079,8 @@
       <c r="G45">
         <v>71</v>
       </c>
-      <c r="H45">
-        <v>1</v>
+      <c r="H45" t="str">
+        <v>US</v>
       </c>
       <c r="I45" t="s">
         <v>40</v>
@@ -3116,8 +3116,8 @@
       <c r="G46">
         <v>71</v>
       </c>
-      <c r="H46">
-        <v>1</v>
+      <c r="H46" t="str">
+        <v>US</v>
       </c>
       <c r="I46" t="s">
         <v>41</v>
@@ -3153,8 +3153,8 @@
       <c r="G47">
         <v>71</v>
       </c>
-      <c r="H47">
-        <v>1</v>
+      <c r="H47" t="str">
+        <v>US</v>
       </c>
       <c r="I47" t="s">
         <v>6</v>
@@ -3190,8 +3190,8 @@
       <c r="G48">
         <v>71</v>
       </c>
-      <c r="H48">
-        <v>1</v>
+      <c r="H48" t="str">
+        <v>US</v>
       </c>
       <c r="I48" t="s">
         <v>42</v>
@@ -3227,8 +3227,8 @@
       <c r="G49">
         <v>71</v>
       </c>
-      <c r="H49">
-        <v>1</v>
+      <c r="H49" t="str">
+        <v>US</v>
       </c>
       <c r="I49" t="s">
         <v>5</v>
@@ -3264,8 +3264,8 @@
       <c r="G50">
         <v>71</v>
       </c>
-      <c r="H50">
-        <v>1</v>
+      <c r="H50" t="str">
+        <v>US</v>
       </c>
       <c r="I50" t="s">
         <v>7</v>
@@ -3301,8 +3301,8 @@
       <c r="G51">
         <v>71</v>
       </c>
-      <c r="H51">
-        <v>1</v>
+      <c r="H51" t="str">
+        <v>US</v>
       </c>
       <c r="I51" t="s">
         <v>43</v>
@@ -3338,8 +3338,8 @@
       <c r="G52">
         <v>71</v>
       </c>
-      <c r="H52">
-        <v>1</v>
+      <c r="H52" t="str">
+        <v>US</v>
       </c>
       <c r="I52" t="s">
         <v>44</v>
@@ -3375,8 +3375,8 @@
       <c r="G53">
         <v>71</v>
       </c>
-      <c r="H53">
-        <v>1</v>
+      <c r="H53" t="str">
+        <v>US</v>
       </c>
       <c r="I53" t="s">
         <v>45</v>
@@ -3412,8 +3412,8 @@
       <c r="G54">
         <v>71</v>
       </c>
-      <c r="H54">
-        <v>1</v>
+      <c r="H54" t="str">
+        <v>US</v>
       </c>
       <c r="I54" t="s">
         <v>46</v>
@@ -3449,8 +3449,8 @@
       <c r="G55">
         <v>71</v>
       </c>
-      <c r="H55">
-        <v>1</v>
+      <c r="H55" t="str">
+        <v>US</v>
       </c>
       <c r="I55" t="s">
         <v>47</v>
@@ -3486,8 +3486,8 @@
       <c r="G56">
         <v>71</v>
       </c>
-      <c r="H56">
-        <v>1</v>
+      <c r="H56" t="str">
+        <v>US</v>
       </c>
       <c r="I56" t="s">
         <v>48</v>
@@ -3523,8 +3523,8 @@
       <c r="G57">
         <v>71</v>
       </c>
-      <c r="H57">
-        <v>1</v>
+      <c r="H57" t="str">
+        <v>US</v>
       </c>
       <c r="I57" t="s">
         <v>49</v>
@@ -3560,8 +3560,8 @@
       <c r="G58">
         <v>71</v>
       </c>
-      <c r="H58">
-        <v>1</v>
+      <c r="H58" t="str">
+        <v>US</v>
       </c>
       <c r="I58" t="s">
         <v>50</v>
@@ -3597,8 +3597,8 @@
       <c r="G59">
         <v>71</v>
       </c>
-      <c r="H59">
-        <v>2</v>
+      <c r="H59" t="str">
+        <v>Europe</v>
       </c>
       <c r="I59" t="s">
         <v>51</v>
@@ -3634,8 +3634,8 @@
       <c r="G60">
         <v>71</v>
       </c>
-      <c r="H60">
-        <v>2</v>
+      <c r="H60" t="str">
+        <v>Europe</v>
       </c>
       <c r="I60" t="s">
         <v>52</v>
@@ -3671,8 +3671,8 @@
       <c r="G61">
         <v>71</v>
       </c>
-      <c r="H61">
-        <v>2</v>
+      <c r="H61" t="str">
+        <v>Europe</v>
       </c>
       <c r="I61" t="s">
         <v>53</v>
@@ -3708,8 +3708,8 @@
       <c r="G62">
         <v>71</v>
       </c>
-      <c r="H62">
-        <v>3</v>
+      <c r="H62" t="str">
+        <v>Asia</v>
       </c>
       <c r="I62" t="s">
         <v>54</v>
@@ -3745,8 +3745,8 @@
       <c r="G63">
         <v>71</v>
       </c>
-      <c r="H63">
-        <v>3</v>
+      <c r="H63" t="str">
+        <v>Asia</v>
       </c>
       <c r="I63" t="s">
         <v>55</v>
@@ -3782,8 +3782,8 @@
       <c r="G64">
         <v>71</v>
       </c>
-      <c r="H64">
-        <v>2</v>
+      <c r="H64" t="str">
+        <v>Europe</v>
       </c>
       <c r="I64" t="s">
         <v>56</v>
@@ -3819,8 +3819,8 @@
       <c r="G65">
         <v>71</v>
       </c>
-      <c r="H65">
-        <v>1</v>
+      <c r="H65" t="str">
+        <v>US</v>
       </c>
       <c r="I65" t="s">
         <v>57</v>
@@ -3856,8 +3856,8 @@
       <c r="G66">
         <v>72</v>
       </c>
-      <c r="H66">
-        <v>3</v>
+      <c r="H66" t="str">
+        <v>Asia</v>
       </c>
       <c r="I66" t="s">
         <v>58</v>
@@ -3893,8 +3893,8 @@
       <c r="G67">
         <v>72</v>
       </c>
-      <c r="H67">
-        <v>1</v>
+      <c r="H67" t="str">
+        <v>US</v>
       </c>
       <c r="I67" t="s">
         <v>59</v>
@@ -3930,8 +3930,8 @@
       <c r="G68">
         <v>72</v>
       </c>
-      <c r="H68">
-        <v>2</v>
+      <c r="H68" t="str">
+        <v>Europe</v>
       </c>
       <c r="I68" t="s">
         <v>60</v>
@@ -3967,8 +3967,8 @@
       <c r="G69">
         <v>72</v>
       </c>
-      <c r="H69">
-        <v>1</v>
+      <c r="H69" t="str">
+        <v>US</v>
       </c>
       <c r="I69" t="s">
         <v>61</v>
@@ -4004,8 +4004,8 @@
       <c r="G70">
         <v>72</v>
       </c>
-      <c r="H70">
-        <v>1</v>
+      <c r="H70" t="str">
+        <v>US</v>
       </c>
       <c r="I70" t="s">
         <v>62</v>
@@ -4041,8 +4041,8 @@
       <c r="G71">
         <v>72</v>
       </c>
-      <c r="H71">
-        <v>1</v>
+      <c r="H71" t="str">
+        <v>US</v>
       </c>
       <c r="I71" t="s">
         <v>6</v>
@@ -4078,8 +4078,8 @@
       <c r="G72">
         <v>72</v>
       </c>
-      <c r="H72">
-        <v>1</v>
+      <c r="H72" t="str">
+        <v>US</v>
       </c>
       <c r="I72" t="s">
         <v>8</v>
@@ -4115,8 +4115,8 @@
       <c r="G73">
         <v>72</v>
       </c>
-      <c r="H73">
-        <v>1</v>
+      <c r="H73" t="str">
+        <v>US</v>
       </c>
       <c r="I73" t="s">
         <v>7</v>
@@ -4152,8 +4152,8 @@
       <c r="G74">
         <v>72</v>
       </c>
-      <c r="H74">
-        <v>1</v>
+      <c r="H74" t="str">
+        <v>US</v>
       </c>
       <c r="I74" t="s">
         <v>5</v>
@@ -4189,8 +4189,8 @@
       <c r="G75">
         <v>72</v>
       </c>
-      <c r="H75">
-        <v>1</v>
+      <c r="H75" t="str">
+        <v>US</v>
       </c>
       <c r="I75" t="s">
         <v>63</v>
@@ -4226,8 +4226,8 @@
       <c r="G76">
         <v>72</v>
       </c>
-      <c r="H76">
-        <v>1</v>
+      <c r="H76" t="str">
+        <v>US</v>
       </c>
       <c r="I76" t="s">
         <v>64</v>
@@ -4263,8 +4263,8 @@
       <c r="G77">
         <v>72</v>
       </c>
-      <c r="H77">
-        <v>1</v>
+      <c r="H77" t="str">
+        <v>US</v>
       </c>
       <c r="I77" t="s">
         <v>65</v>
@@ -4300,8 +4300,8 @@
       <c r="G78">
         <v>72</v>
       </c>
-      <c r="H78">
-        <v>1</v>
+      <c r="H78" t="str">
+        <v>US</v>
       </c>
       <c r="I78" t="s">
         <v>66</v>
@@ -4337,8 +4337,8 @@
       <c r="G79">
         <v>72</v>
       </c>
-      <c r="H79">
-        <v>1</v>
+      <c r="H79" t="str">
+        <v>US</v>
       </c>
       <c r="I79" t="s">
         <v>67</v>
@@ -4374,8 +4374,8 @@
       <c r="G80">
         <v>72</v>
       </c>
-      <c r="H80">
-        <v>3</v>
+      <c r="H80" t="str">
+        <v>Asia</v>
       </c>
       <c r="I80" t="s">
         <v>68</v>
@@ -4411,8 +4411,8 @@
       <c r="G81">
         <v>72</v>
       </c>
-      <c r="H81">
-        <v>1</v>
+      <c r="H81" t="str">
+        <v>US</v>
       </c>
       <c r="I81" t="s">
         <v>69</v>
@@ -4448,8 +4448,8 @@
       <c r="G82">
         <v>72</v>
       </c>
-      <c r="H82">
-        <v>1</v>
+      <c r="H82" t="str">
+        <v>US</v>
       </c>
       <c r="I82" t="s">
         <v>11</v>
@@ -4485,8 +4485,8 @@
       <c r="G83">
         <v>72</v>
       </c>
-      <c r="H83">
-        <v>1</v>
+      <c r="H83" t="str">
+        <v>US</v>
       </c>
       <c r="I83" t="s">
         <v>70</v>
@@ -4522,8 +4522,8 @@
       <c r="G84">
         <v>72</v>
       </c>
-      <c r="H84">
-        <v>1</v>
+      <c r="H84" t="str">
+        <v>US</v>
       </c>
       <c r="I84" t="s">
         <v>71</v>
@@ -4559,8 +4559,8 @@
       <c r="G85">
         <v>72</v>
       </c>
-      <c r="H85">
-        <v>2</v>
+      <c r="H85" t="str">
+        <v>Europe</v>
       </c>
       <c r="I85" t="s">
         <v>72</v>
@@ -4596,8 +4596,8 @@
       <c r="G86">
         <v>72</v>
       </c>
-      <c r="H86">
-        <v>2</v>
+      <c r="H86" t="str">
+        <v>Europe</v>
       </c>
       <c r="I86" t="s">
         <v>73</v>
@@ -4633,8 +4633,8 @@
       <c r="G87">
         <v>72</v>
       </c>
-      <c r="H87">
-        <v>2</v>
+      <c r="H87" t="str">
+        <v>Europe</v>
       </c>
       <c r="I87" t="s">
         <v>74</v>
@@ -4670,8 +4670,8 @@
       <c r="G88">
         <v>72</v>
       </c>
-      <c r="H88">
-        <v>2</v>
+      <c r="H88" t="str">
+        <v>Europe</v>
       </c>
       <c r="I88" t="s">
         <v>75</v>
@@ -4707,8 +4707,8 @@
       <c r="G89">
         <v>72</v>
       </c>
-      <c r="H89">
-        <v>1</v>
+      <c r="H89" t="str">
+        <v>US</v>
       </c>
       <c r="I89" t="s">
         <v>76</v>
@@ -4744,8 +4744,8 @@
       <c r="G90">
         <v>72</v>
       </c>
-      <c r="H90">
-        <v>3</v>
+      <c r="H90" t="str">
+        <v>Asia</v>
       </c>
       <c r="I90" t="s">
         <v>77</v>
@@ -4781,8 +4781,8 @@
       <c r="G91">
         <v>72</v>
       </c>
-      <c r="H91">
-        <v>3</v>
+      <c r="H91" t="str">
+        <v>Asia</v>
       </c>
       <c r="I91" t="s">
         <v>78</v>
@@ -4818,8 +4818,8 @@
       <c r="G92">
         <v>72</v>
       </c>
-      <c r="H92">
-        <v>1</v>
+      <c r="H92" t="str">
+        <v>US</v>
       </c>
       <c r="I92" t="s">
         <v>79</v>
@@ -4855,8 +4855,8 @@
       <c r="G93">
         <v>72</v>
       </c>
-      <c r="H93">
-        <v>3</v>
+      <c r="H93" t="str">
+        <v>Asia</v>
       </c>
       <c r="I93" t="s">
         <v>80</v>
@@ -4892,8 +4892,8 @@
       <c r="G94">
         <v>73</v>
       </c>
-      <c r="H94">
-        <v>1</v>
+      <c r="H94" t="str">
+        <v>US</v>
       </c>
       <c r="I94" t="s">
         <v>81</v>
@@ -4929,8 +4929,8 @@
       <c r="G95">
         <v>73</v>
       </c>
-      <c r="H95">
-        <v>1</v>
+      <c r="H95" t="str">
+        <v>US</v>
       </c>
       <c r="I95" t="s">
         <v>41</v>
@@ -4966,8 +4966,8 @@
       <c r="G96">
         <v>73</v>
       </c>
-      <c r="H96">
-        <v>1</v>
+      <c r="H96" t="str">
+        <v>US</v>
       </c>
       <c r="I96" t="s">
         <v>82</v>
@@ -5003,8 +5003,8 @@
       <c r="G97">
         <v>73</v>
       </c>
-      <c r="H97">
-        <v>1</v>
+      <c r="H97" t="str">
+        <v>US</v>
       </c>
       <c r="I97" t="s">
         <v>83</v>
@@ -5040,8 +5040,8 @@
       <c r="G98">
         <v>73</v>
       </c>
-      <c r="H98">
-        <v>1</v>
+      <c r="H98" t="str">
+        <v>US</v>
       </c>
       <c r="I98" t="s">
         <v>84</v>
@@ -5077,8 +5077,8 @@
       <c r="G99">
         <v>73</v>
       </c>
-      <c r="H99">
-        <v>1</v>
+      <c r="H99" t="str">
+        <v>US</v>
       </c>
       <c r="I99" t="s">
         <v>85</v>
@@ -5114,8 +5114,8 @@
       <c r="G100">
         <v>73</v>
       </c>
-      <c r="H100">
-        <v>1</v>
+      <c r="H100" t="str">
+        <v>US</v>
       </c>
       <c r="I100" t="s">
         <v>86</v>
@@ -5151,8 +5151,8 @@
       <c r="G101">
         <v>73</v>
       </c>
-      <c r="H101">
-        <v>1</v>
+      <c r="H101" t="str">
+        <v>US</v>
       </c>
       <c r="I101" t="s">
         <v>87</v>
@@ -5188,8 +5188,8 @@
       <c r="G102">
         <v>73</v>
       </c>
-      <c r="H102">
-        <v>1</v>
+      <c r="H102" t="str">
+        <v>US</v>
       </c>
       <c r="I102" t="s">
         <v>88</v>
@@ -5225,8 +5225,8 @@
       <c r="G103">
         <v>73</v>
       </c>
-      <c r="H103">
-        <v>1</v>
+      <c r="H103" t="str">
+        <v>US</v>
       </c>
       <c r="I103" t="s">
         <v>89</v>
@@ -5262,8 +5262,8 @@
       <c r="G104">
         <v>73</v>
       </c>
-      <c r="H104">
-        <v>1</v>
+      <c r="H104" t="str">
+        <v>US</v>
       </c>
       <c r="I104" t="s">
         <v>90</v>
@@ -5299,8 +5299,8 @@
       <c r="G105">
         <v>73</v>
       </c>
-      <c r="H105">
-        <v>1</v>
+      <c r="H105" t="str">
+        <v>US</v>
       </c>
       <c r="I105" t="s">
         <v>91</v>
@@ -5336,8 +5336,8 @@
       <c r="G106">
         <v>73</v>
       </c>
-      <c r="H106">
-        <v>1</v>
+      <c r="H106" t="str">
+        <v>US</v>
       </c>
       <c r="I106" t="s">
         <v>92</v>
@@ -5373,8 +5373,8 @@
       <c r="G107">
         <v>73</v>
       </c>
-      <c r="H107">
-        <v>1</v>
+      <c r="H107" t="str">
+        <v>US</v>
       </c>
       <c r="I107" t="s">
         <v>93</v>
@@ -5410,8 +5410,8 @@
       <c r="G108">
         <v>73</v>
       </c>
-      <c r="H108">
-        <v>1</v>
+      <c r="H108" t="str">
+        <v>US</v>
       </c>
       <c r="I108" t="s">
         <v>22</v>
@@ -5447,8 +5447,8 @@
       <c r="G109">
         <v>73</v>
       </c>
-      <c r="H109">
-        <v>1</v>
+      <c r="H109" t="str">
+        <v>US</v>
       </c>
       <c r="I109" t="s">
         <v>23</v>
@@ -5484,8 +5484,8 @@
       <c r="G110">
         <v>73</v>
       </c>
-      <c r="H110">
-        <v>1</v>
+      <c r="H110" t="str">
+        <v>US</v>
       </c>
       <c r="I110" t="s">
         <v>21</v>
@@ -5521,8 +5521,8 @@
       <c r="G111">
         <v>73</v>
       </c>
-      <c r="H111">
-        <v>2</v>
+      <c r="H111" t="str">
+        <v>Europe</v>
       </c>
       <c r="I111" t="s">
         <v>94</v>
@@ -5558,8 +5558,8 @@
       <c r="G112">
         <v>73</v>
       </c>
-      <c r="H112">
-        <v>1</v>
+      <c r="H112" t="str">
+        <v>US</v>
       </c>
       <c r="I112" t="s">
         <v>6</v>
@@ -5595,8 +5595,8 @@
       <c r="G113">
         <v>73</v>
       </c>
-      <c r="H113">
-        <v>1</v>
+      <c r="H113" t="str">
+        <v>US</v>
       </c>
       <c r="I113" t="s">
         <v>95</v>
@@ -5632,8 +5632,8 @@
       <c r="G114">
         <v>73</v>
       </c>
-      <c r="H114">
-        <v>1</v>
+      <c r="H114" t="str">
+        <v>US</v>
       </c>
       <c r="I114" t="s">
         <v>96</v>
@@ -5669,8 +5669,8 @@
       <c r="G115">
         <v>73</v>
       </c>
-      <c r="H115">
-        <v>1</v>
+      <c r="H115" t="str">
+        <v>US</v>
       </c>
       <c r="I115" t="s">
         <v>97</v>
@@ -5706,8 +5706,8 @@
       <c r="G116">
         <v>73</v>
       </c>
-      <c r="H116">
-        <v>1</v>
+      <c r="H116" t="str">
+        <v>US</v>
       </c>
       <c r="I116" t="s">
         <v>30</v>
@@ -5743,8 +5743,8 @@
       <c r="G117">
         <v>73</v>
       </c>
-      <c r="H117">
-        <v>3</v>
+      <c r="H117" t="str">
+        <v>Asia</v>
       </c>
       <c r="I117" t="s">
         <v>98</v>
@@ -5780,8 +5780,8 @@
       <c r="G118">
         <v>73</v>
       </c>
-      <c r="H118">
-        <v>1</v>
+      <c r="H118" t="str">
+        <v>US</v>
       </c>
       <c r="I118" t="s">
         <v>61</v>
@@ -5817,8 +5817,8 @@
       <c r="G119">
         <v>73</v>
       </c>
-      <c r="H119">
-        <v>3</v>
+      <c r="H119" t="str">
+        <v>Asia</v>
       </c>
       <c r="I119" t="s">
         <v>99</v>
@@ -5854,8 +5854,8 @@
       <c r="G120">
         <v>73</v>
       </c>
-      <c r="H120">
-        <v>3</v>
+      <c r="H120" t="str">
+        <v>Asia</v>
       </c>
       <c r="I120" t="s">
         <v>100</v>
@@ -5891,8 +5891,8 @@
       <c r="G121">
         <v>73</v>
       </c>
-      <c r="H121">
-        <v>1</v>
+      <c r="H121" t="str">
+        <v>US</v>
       </c>
       <c r="I121" t="s">
         <v>37</v>
@@ -5928,8 +5928,8 @@
       <c r="G122">
         <v>73</v>
       </c>
-      <c r="H122">
-        <v>1</v>
+      <c r="H122" t="str">
+        <v>US</v>
       </c>
       <c r="I122" t="s">
         <v>101</v>
@@ -5965,8 +5965,8 @@
       <c r="G123">
         <v>73</v>
       </c>
-      <c r="H123">
-        <v>2</v>
+      <c r="H123" t="str">
+        <v>Europe</v>
       </c>
       <c r="I123" t="s">
         <v>102</v>
@@ -6002,8 +6002,8 @@
       <c r="G124">
         <v>73</v>
       </c>
-      <c r="H124">
-        <v>1</v>
+      <c r="H124" t="str">
+        <v>US</v>
       </c>
       <c r="I124" t="s">
         <v>103</v>
@@ -6039,8 +6039,8 @@
       <c r="G125">
         <v>73</v>
       </c>
-      <c r="H125">
-        <v>1</v>
+      <c r="H125" t="str">
+        <v>US</v>
       </c>
       <c r="I125" t="s">
         <v>104</v>
@@ -6076,8 +6076,8 @@
       <c r="G126">
         <v>73</v>
       </c>
-      <c r="H126">
-        <v>2</v>
+      <c r="H126" t="str">
+        <v>Europe</v>
       </c>
       <c r="I126" t="s">
         <v>105</v>
@@ -6113,8 +6113,8 @@
       <c r="G127">
         <v>73</v>
       </c>
-      <c r="H127">
-        <v>2</v>
+      <c r="H127" t="str">
+        <v>Europe</v>
       </c>
       <c r="I127" t="s">
         <v>106</v>
@@ -6150,8 +6150,8 @@
       <c r="G128">
         <v>73</v>
       </c>
-      <c r="H128">
-        <v>2</v>
+      <c r="H128" t="str">
+        <v>Europe</v>
       </c>
       <c r="I128" t="s">
         <v>107</v>
@@ -6187,8 +6187,8 @@
       <c r="G129">
         <v>73</v>
       </c>
-      <c r="H129">
-        <v>2</v>
+      <c r="H129" t="str">
+        <v>Europe</v>
       </c>
       <c r="I129" t="s">
         <v>108</v>
@@ -6224,8 +6224,8 @@
       <c r="G130">
         <v>73</v>
       </c>
-      <c r="H130">
-        <v>1</v>
+      <c r="H130" t="str">
+        <v>US</v>
       </c>
       <c r="I130" t="s">
         <v>109</v>
@@ -6261,8 +6261,8 @@
       <c r="G131">
         <v>73</v>
       </c>
-      <c r="H131">
-        <v>2</v>
+      <c r="H131" t="str">
+        <v>Europe</v>
       </c>
       <c r="I131" t="s">
         <v>110</v>
@@ -6298,8 +6298,8 @@
       <c r="G132">
         <v>73</v>
       </c>
-      <c r="H132">
-        <v>3</v>
+      <c r="H132" t="str">
+        <v>Asia</v>
       </c>
       <c r="I132" t="s">
         <v>111</v>
@@ -6335,8 +6335,8 @@
       <c r="G133">
         <v>73</v>
       </c>
-      <c r="H133">
-        <v>1</v>
+      <c r="H133" t="str">
+        <v>US</v>
       </c>
       <c r="I133" t="s">
         <v>112</v>
@@ -6372,8 +6372,8 @@
       <c r="G134">
         <v>74</v>
       </c>
-      <c r="H134">
-        <v>1</v>
+      <c r="H134" t="str">
+        <v>US</v>
       </c>
       <c r="I134" t="s">
         <v>21</v>
@@ -6409,8 +6409,8 @@
       <c r="G135">
         <v>74</v>
       </c>
-      <c r="H135">
-        <v>1</v>
+      <c r="H135" t="str">
+        <v>US</v>
       </c>
       <c r="I135" t="s">
         <v>23</v>
@@ -6446,8 +6446,8 @@
       <c r="G136">
         <v>74</v>
       </c>
-      <c r="H136">
-        <v>1</v>
+      <c r="H136" t="str">
+        <v>US</v>
       </c>
       <c r="I136" t="s">
         <v>22</v>
@@ -6483,8 +6483,8 @@
       <c r="G137">
         <v>74</v>
       </c>
-      <c r="H137">
-        <v>1</v>
+      <c r="H137" t="str">
+        <v>US</v>
       </c>
       <c r="I137" t="s">
         <v>113</v>
@@ -6520,8 +6520,8 @@
       <c r="G138">
         <v>74</v>
       </c>
-      <c r="H138">
-        <v>3</v>
+      <c r="H138" t="str">
+        <v>Asia</v>
       </c>
       <c r="I138" t="s">
         <v>114</v>
@@ -6557,8 +6557,8 @@
       <c r="G139">
         <v>74</v>
       </c>
-      <c r="H139">
-        <v>1</v>
+      <c r="H139" t="str">
+        <v>US</v>
       </c>
       <c r="I139" t="s">
         <v>37</v>
@@ -6594,8 +6594,8 @@
       <c r="G140">
         <v>74</v>
       </c>
-      <c r="H140">
-        <v>3</v>
+      <c r="H140" t="str">
+        <v>Asia</v>
       </c>
       <c r="I140" t="s">
         <v>54</v>
@@ -6631,8 +6631,8 @@
       <c r="G141">
         <v>74</v>
       </c>
-      <c r="H141">
-        <v>1</v>
+      <c r="H141" t="str">
+        <v>US</v>
       </c>
       <c r="I141" t="s">
         <v>61</v>
@@ -6668,8 +6668,8 @@
       <c r="G142">
         <v>74</v>
       </c>
-      <c r="H142">
-        <v>1</v>
+      <c r="H142" t="str">
+        <v>US</v>
       </c>
       <c r="I142" t="s">
         <v>115</v>
@@ -6705,8 +6705,8 @@
       <c r="G143">
         <v>74</v>
       </c>
-      <c r="H143">
-        <v>1</v>
+      <c r="H143" t="str">
+        <v>US</v>
       </c>
       <c r="I143" t="s">
         <v>41</v>
@@ -6742,8 +6742,8 @@
       <c r="G144">
         <v>74</v>
       </c>
-      <c r="H144">
-        <v>1</v>
+      <c r="H144" t="str">
+        <v>US</v>
       </c>
       <c r="I144" t="s">
         <v>116</v>
@@ -6779,8 +6779,8 @@
       <c r="G145">
         <v>74</v>
       </c>
-      <c r="H145">
-        <v>1</v>
+      <c r="H145" t="str">
+        <v>US</v>
       </c>
       <c r="I145" t="s">
         <v>83</v>
@@ -6816,8 +6816,8 @@
       <c r="G146">
         <v>74</v>
       </c>
-      <c r="H146">
-        <v>1</v>
+      <c r="H146" t="str">
+        <v>US</v>
       </c>
       <c r="I146" t="s">
         <v>117</v>
@@ -6853,8 +6853,8 @@
       <c r="G147">
         <v>74</v>
       </c>
-      <c r="H147">
-        <v>1</v>
+      <c r="H147" t="str">
+        <v>US</v>
       </c>
       <c r="I147" t="s">
         <v>118</v>
@@ -6890,8 +6890,8 @@
       <c r="G148">
         <v>74</v>
       </c>
-      <c r="H148">
-        <v>1</v>
+      <c r="H148" t="str">
+        <v>US</v>
       </c>
       <c r="I148" t="s">
         <v>70</v>
@@ -6927,8 +6927,8 @@
       <c r="G149">
         <v>74</v>
       </c>
-      <c r="H149">
-        <v>1</v>
+      <c r="H149" t="str">
+        <v>US</v>
       </c>
       <c r="I149" t="s">
         <v>69</v>
@@ -6964,8 +6964,8 @@
       <c r="G150">
         <v>74</v>
       </c>
-      <c r="H150">
-        <v>2</v>
+      <c r="H150" t="str">
+        <v>Europe</v>
       </c>
       <c r="I150" t="s">
         <v>119</v>
@@ -7001,8 +7001,8 @@
       <c r="G151">
         <v>74</v>
       </c>
-      <c r="H151">
-        <v>2</v>
+      <c r="H151" t="str">
+        <v>Europe</v>
       </c>
       <c r="I151" t="s">
         <v>120</v>
@@ -7038,8 +7038,8 @@
       <c r="G152">
         <v>74</v>
       </c>
-      <c r="H152">
-        <v>2</v>
+      <c r="H152" t="str">
+        <v>Europe</v>
       </c>
       <c r="I152" t="s">
         <v>106</v>
@@ -7075,8 +7075,8 @@
       <c r="G153">
         <v>74</v>
       </c>
-      <c r="H153">
-        <v>3</v>
+      <c r="H153" t="str">
+        <v>Asia</v>
       </c>
       <c r="I153" t="s">
         <v>36</v>
@@ -7112,8 +7112,8 @@
       <c r="G154">
         <v>74</v>
       </c>
-      <c r="H154">
-        <v>3</v>
+      <c r="H154" t="str">
+        <v>Asia</v>
       </c>
       <c r="I154" t="s">
         <v>121</v>
@@ -7149,8 +7149,8 @@
       <c r="G155">
         <v>74</v>
       </c>
-      <c r="H155">
-        <v>1</v>
+      <c r="H155" t="str">
+        <v>US</v>
       </c>
       <c r="I155" t="s">
         <v>122</v>
@@ -7186,8 +7186,8 @@
       <c r="G156">
         <v>74</v>
       </c>
-      <c r="H156">
-        <v>2</v>
+      <c r="H156" t="str">
+        <v>Europe</v>
       </c>
       <c r="I156" t="s">
         <v>105</v>
@@ -7223,8 +7223,8 @@
       <c r="G157">
         <v>74</v>
       </c>
-      <c r="H157">
-        <v>2</v>
+      <c r="H157" t="str">
+        <v>Europe</v>
       </c>
       <c r="I157" t="s">
         <v>123</v>
@@ -7260,8 +7260,8 @@
       <c r="G158">
         <v>74</v>
       </c>
-      <c r="H158">
-        <v>3</v>
+      <c r="H158" t="str">
+        <v>Asia</v>
       </c>
       <c r="I158" t="s">
         <v>124</v>
@@ -7297,8 +7297,8 @@
       <c r="G159">
         <v>74</v>
       </c>
-      <c r="H159">
-        <v>3</v>
+      <c r="H159" t="str">
+        <v>Asia</v>
       </c>
       <c r="I159" t="s">
         <v>125</v>
@@ -7334,8 +7334,8 @@
       <c r="G160">
         <v>74</v>
       </c>
-      <c r="H160">
-        <v>2</v>
+      <c r="H160" t="str">
+        <v>Europe</v>
       </c>
       <c r="I160" t="s">
         <v>126</v>
@@ -7371,8 +7371,8 @@
       <c r="G161">
         <v>75</v>
       </c>
-      <c r="H161">
-        <v>1</v>
+      <c r="H161" t="str">
+        <v>US</v>
       </c>
       <c r="I161" t="s">
         <v>127</v>
@@ -7408,8 +7408,8 @@
       <c r="G162">
         <v>75</v>
       </c>
-      <c r="H162">
-        <v>1</v>
+      <c r="H162" t="str">
+        <v>US</v>
       </c>
       <c r="I162" t="s">
         <v>113</v>
@@ -7445,8 +7445,8 @@
       <c r="G163">
         <v>75</v>
       </c>
-      <c r="H163">
-        <v>1</v>
+      <c r="H163" t="str">
+        <v>US</v>
       </c>
       <c r="I163" t="s">
         <v>128</v>
@@ -7482,8 +7482,8 @@
       <c r="G164">
         <v>75</v>
       </c>
-      <c r="H164">
-        <v>1</v>
+      <c r="H164" t="str">
+        <v>US</v>
       </c>
       <c r="I164" t="s">
         <v>23</v>
@@ -7519,8 +7519,8 @@
       <c r="G165">
         <v>75</v>
       </c>
-      <c r="H165">
-        <v>1</v>
+      <c r="H165" t="str">
+        <v>US</v>
       </c>
       <c r="I165" t="s">
         <v>8</v>
@@ -7556,8 +7556,8 @@
       <c r="G166">
         <v>75</v>
       </c>
-      <c r="H166">
-        <v>1</v>
+      <c r="H166" t="str">
+        <v>US</v>
       </c>
       <c r="I166" t="s">
         <v>129</v>
@@ -7593,8 +7593,8 @@
       <c r="G167">
         <v>75</v>
       </c>
-      <c r="H167">
-        <v>1</v>
+      <c r="H167" t="str">
+        <v>US</v>
       </c>
       <c r="I167" t="s">
         <v>130</v>
@@ -7630,8 +7630,8 @@
       <c r="G168">
         <v>75</v>
       </c>
-      <c r="H168">
-        <v>1</v>
+      <c r="H168" t="str">
+        <v>US</v>
       </c>
       <c r="I168" t="s">
         <v>87</v>
@@ -7667,8 +7667,8 @@
       <c r="G169">
         <v>75</v>
       </c>
-      <c r="H169">
-        <v>1</v>
+      <c r="H169" t="str">
+        <v>US</v>
       </c>
       <c r="I169" t="s">
         <v>131</v>
@@ -7704,8 +7704,8 @@
       <c r="G170">
         <v>75</v>
       </c>
-      <c r="H170">
-        <v>1</v>
+      <c r="H170" t="str">
+        <v>US</v>
       </c>
       <c r="I170" t="s">
         <v>132</v>
@@ -7741,8 +7741,8 @@
       <c r="G171">
         <v>75</v>
       </c>
-      <c r="H171">
-        <v>1</v>
+      <c r="H171" t="str">
+        <v>US</v>
       </c>
       <c r="I171" t="s">
         <v>41</v>
@@ -7778,8 +7778,8 @@
       <c r="G172">
         <v>75</v>
       </c>
-      <c r="H172">
-        <v>1</v>
+      <c r="H172" t="str">
+        <v>US</v>
       </c>
       <c r="I172" t="s">
         <v>133</v>
@@ -7815,8 +7815,8 @@
       <c r="G173">
         <v>75</v>
       </c>
-      <c r="H173">
-        <v>1</v>
+      <c r="H173" t="str">
+        <v>US</v>
       </c>
       <c r="I173" t="s">
         <v>134</v>
@@ -7852,8 +7852,8 @@
       <c r="G174">
         <v>75</v>
       </c>
-      <c r="H174">
-        <v>1</v>
+      <c r="H174" t="str">
+        <v>US</v>
       </c>
       <c r="I174" t="s">
         <v>135</v>
@@ -7889,8 +7889,8 @@
       <c r="G175">
         <v>75</v>
       </c>
-      <c r="H175">
-        <v>1</v>
+      <c r="H175" t="str">
+        <v>US</v>
       </c>
       <c r="I175" t="s">
         <v>136</v>
@@ -7926,8 +7926,8 @@
       <c r="G176">
         <v>75</v>
       </c>
-      <c r="H176">
-        <v>3</v>
+      <c r="H176" t="str">
+        <v>Asia</v>
       </c>
       <c r="I176" t="s">
         <v>137</v>
@@ -7963,8 +7963,8 @@
       <c r="G177">
         <v>75</v>
       </c>
-      <c r="H177">
-        <v>1</v>
+      <c r="H177" t="str">
+        <v>US</v>
       </c>
       <c r="I177" t="s">
         <v>37</v>
@@ -8000,8 +8000,8 @@
       <c r="G178">
         <v>75</v>
       </c>
-      <c r="H178">
-        <v>1</v>
+      <c r="H178" t="str">
+        <v>US</v>
       </c>
       <c r="I178" t="s">
         <v>30</v>
@@ -8037,8 +8037,8 @@
       <c r="G179">
         <v>75</v>
       </c>
-      <c r="H179">
-        <v>1</v>
+      <c r="H179" t="str">
+        <v>US</v>
       </c>
       <c r="I179" t="s">
         <v>138</v>
@@ -8074,8 +8074,8 @@
       <c r="G180">
         <v>75</v>
       </c>
-      <c r="H180">
-        <v>3</v>
+      <c r="H180" t="str">
+        <v>Asia</v>
       </c>
       <c r="I180" t="s">
         <v>36</v>
@@ -8111,8 +8111,8 @@
       <c r="G181">
         <v>75</v>
       </c>
-      <c r="H181">
-        <v>2</v>
+      <c r="H181" t="str">
+        <v>Europe</v>
       </c>
       <c r="I181" t="s">
         <v>120</v>
@@ -8148,8 +8148,8 @@
       <c r="G182">
         <v>75</v>
       </c>
-      <c r="H182">
-        <v>3</v>
+      <c r="H182" t="str">
+        <v>Asia</v>
       </c>
       <c r="I182" t="s">
         <v>121</v>
@@ -8185,8 +8185,8 @@
       <c r="G183">
         <v>75</v>
       </c>
-      <c r="H183">
-        <v>1</v>
+      <c r="H183" t="str">
+        <v>US</v>
       </c>
       <c r="I183" t="s">
         <v>37</v>
@@ -8222,8 +8222,8 @@
       <c r="G184">
         <v>75</v>
       </c>
-      <c r="H184">
-        <v>2</v>
+      <c r="H184" t="str">
+        <v>Europe</v>
       </c>
       <c r="I184" t="s">
         <v>139</v>
@@ -8259,8 +8259,8 @@
       <c r="G185">
         <v>75</v>
       </c>
-      <c r="H185">
-        <v>1</v>
+      <c r="H185" t="str">
+        <v>US</v>
       </c>
       <c r="I185" t="s">
         <v>140</v>
@@ -8296,8 +8296,8 @@
       <c r="G186">
         <v>75</v>
       </c>
-      <c r="H186">
-        <v>2</v>
+      <c r="H186" t="str">
+        <v>Europe</v>
       </c>
       <c r="I186" t="s">
         <v>107</v>
@@ -8333,8 +8333,8 @@
       <c r="G187">
         <v>75</v>
       </c>
-      <c r="H187">
-        <v>2</v>
+      <c r="H187" t="str">
+        <v>Europe</v>
       </c>
       <c r="I187" t="s">
         <v>26</v>
@@ -8370,8 +8370,8 @@
       <c r="G188">
         <v>75</v>
       </c>
-      <c r="H188">
-        <v>2</v>
+      <c r="H188" t="str">
+        <v>Europe</v>
       </c>
       <c r="I188" t="s">
         <v>141</v>
@@ -8407,8 +8407,8 @@
       <c r="G189">
         <v>75</v>
       </c>
-      <c r="H189">
-        <v>2</v>
+      <c r="H189" t="str">
+        <v>Europe</v>
       </c>
       <c r="I189" t="s">
         <v>110</v>
@@ -8444,8 +8444,8 @@
       <c r="G190">
         <v>75</v>
       </c>
-      <c r="H190">
-        <v>3</v>
+      <c r="H190" t="str">
+        <v>Asia</v>
       </c>
       <c r="I190" t="s">
         <v>142</v>
@@ -8481,8 +8481,8 @@
       <c r="G191">
         <v>76</v>
       </c>
-      <c r="H191">
-        <v>2</v>
+      <c r="H191" t="str">
+        <v>Europe</v>
       </c>
       <c r="I191" t="s">
         <v>143</v>
@@ -8518,8 +8518,8 @@
       <c r="G192">
         <v>76</v>
       </c>
-      <c r="H192">
-        <v>2</v>
+      <c r="H192" t="str">
+        <v>Europe</v>
       </c>
       <c r="I192" t="s">
         <v>51</v>
@@ -8555,8 +8555,8 @@
       <c r="G193">
         <v>76</v>
       </c>
-      <c r="H193">
-        <v>1</v>
+      <c r="H193" t="str">
+        <v>US</v>
       </c>
       <c r="I193" t="s">
         <v>144</v>
@@ -8592,8 +8592,8 @@
       <c r="G194">
         <v>76</v>
       </c>
-      <c r="H194">
-        <v>1</v>
+      <c r="H194" t="str">
+        <v>US</v>
       </c>
       <c r="I194" t="s">
         <v>122</v>
@@ -8629,8 +8629,8 @@
       <c r="G195">
         <v>76</v>
       </c>
-      <c r="H195">
-        <v>2</v>
+      <c r="H195" t="str">
+        <v>Europe</v>
       </c>
       <c r="I195" t="s">
         <v>145</v>
@@ -8666,8 +8666,8 @@
       <c r="G196">
         <v>76</v>
       </c>
-      <c r="H196">
-        <v>1</v>
+      <c r="H196" t="str">
+        <v>US</v>
       </c>
       <c r="I196" t="s">
         <v>115</v>
@@ -8703,8 +8703,8 @@
       <c r="G197">
         <v>76</v>
       </c>
-      <c r="H197">
-        <v>1</v>
+      <c r="H197" t="str">
+        <v>US</v>
       </c>
       <c r="I197" t="s">
         <v>146</v>
@@ -8740,8 +8740,8 @@
       <c r="G198">
         <v>76</v>
       </c>
-      <c r="H198">
-        <v>1</v>
+      <c r="H198" t="str">
+        <v>US</v>
       </c>
       <c r="I198" t="s">
         <v>41</v>
@@ -8777,8 +8777,8 @@
       <c r="G199">
         <v>76</v>
       </c>
-      <c r="H199">
-        <v>1</v>
+      <c r="H199" t="str">
+        <v>US</v>
       </c>
       <c r="I199" t="s">
         <v>83</v>
@@ -8814,8 +8814,8 @@
       <c r="G200">
         <v>76</v>
       </c>
-      <c r="H200">
-        <v>1</v>
+      <c r="H200" t="str">
+        <v>US</v>
       </c>
       <c r="I200" t="s">
         <v>92</v>
@@ -8851,8 +8851,8 @@
       <c r="G201">
         <v>76</v>
       </c>
-      <c r="H201">
-        <v>1</v>
+      <c r="H201" t="str">
+        <v>US</v>
       </c>
       <c r="I201" t="s">
         <v>113</v>
@@ -8888,8 +8888,8 @@
       <c r="G202">
         <v>76</v>
       </c>
-      <c r="H202">
-        <v>1</v>
+      <c r="H202" t="str">
+        <v>US</v>
       </c>
       <c r="I202" t="s">
         <v>23</v>
@@ -8925,8 +8925,8 @@
       <c r="G203">
         <v>76</v>
       </c>
-      <c r="H203">
-        <v>1</v>
+      <c r="H203" t="str">
+        <v>US</v>
       </c>
       <c r="I203" t="s">
         <v>22</v>
@@ -8962,8 +8962,8 @@
       <c r="G204">
         <v>76</v>
       </c>
-      <c r="H204">
-        <v>1</v>
+      <c r="H204" t="str">
+        <v>US</v>
       </c>
       <c r="I204" t="s">
         <v>147</v>
@@ -8999,8 +8999,8 @@
       <c r="G205">
         <v>76</v>
       </c>
-      <c r="H205">
-        <v>1</v>
+      <c r="H205" t="str">
+        <v>US</v>
       </c>
       <c r="I205" t="s">
         <v>148</v>
@@ -9036,8 +9036,8 @@
       <c r="G206">
         <v>76</v>
       </c>
-      <c r="H206">
-        <v>2</v>
+      <c r="H206" t="str">
+        <v>Europe</v>
       </c>
       <c r="I206" t="s">
         <v>149</v>
@@ -9073,8 +9073,8 @@
       <c r="G207">
         <v>76</v>
       </c>
-      <c r="H207">
-        <v>3</v>
+      <c r="H207" t="str">
+        <v>Asia</v>
       </c>
       <c r="I207" t="s">
         <v>124</v>
@@ -9110,8 +9110,8 @@
       <c r="G208">
         <v>76</v>
       </c>
-      <c r="H208">
-        <v>1</v>
+      <c r="H208" t="str">
+        <v>US</v>
       </c>
       <c r="I208" t="s">
         <v>150</v>
@@ -9147,8 +9147,8 @@
       <c r="G209">
         <v>76</v>
       </c>
-      <c r="H209">
-        <v>1</v>
+      <c r="H209" t="str">
+        <v>US</v>
       </c>
       <c r="I209" t="s">
         <v>151</v>
@@ -9184,8 +9184,8 @@
       <c r="G210">
         <v>76</v>
       </c>
-      <c r="H210">
-        <v>1</v>
+      <c r="H210" t="str">
+        <v>US</v>
       </c>
       <c r="I210" t="s">
         <v>152</v>
@@ -9221,8 +9221,8 @@
       <c r="G211">
         <v>76</v>
       </c>
-      <c r="H211">
-        <v>1</v>
+      <c r="H211" t="str">
+        <v>US</v>
       </c>
       <c r="I211" t="s">
         <v>153</v>
@@ -9258,8 +9258,8 @@
       <c r="G212">
         <v>76</v>
       </c>
-      <c r="H212">
-        <v>2</v>
+      <c r="H212" t="str">
+        <v>Europe</v>
       </c>
       <c r="I212" t="s">
         <v>139</v>
@@ -9295,8 +9295,8 @@
       <c r="G213">
         <v>76</v>
       </c>
-      <c r="H213">
-        <v>3</v>
+      <c r="H213" t="str">
+        <v>Asia</v>
       </c>
       <c r="I213" t="s">
         <v>154</v>
@@ -9332,8 +9332,8 @@
       <c r="G214">
         <v>76</v>
       </c>
-      <c r="H214">
-        <v>3</v>
+      <c r="H214" t="str">
+        <v>Asia</v>
       </c>
       <c r="I214" t="s">
         <v>137</v>
@@ -9369,8 +9369,8 @@
       <c r="G215">
         <v>76</v>
       </c>
-      <c r="H215">
-        <v>1</v>
+      <c r="H215" t="str">
+        <v>US</v>
       </c>
       <c r="I215" t="s">
         <v>37</v>
@@ -9406,8 +9406,8 @@
       <c r="G216">
         <v>76</v>
       </c>
-      <c r="H216">
-        <v>2</v>
+      <c r="H216" t="str">
+        <v>Europe</v>
       </c>
       <c r="I216" t="s">
         <v>155</v>
@@ -9443,8 +9443,8 @@
       <c r="G217">
         <v>76</v>
       </c>
-      <c r="H217">
-        <v>1</v>
+      <c r="H217" t="str">
+        <v>US</v>
       </c>
       <c r="I217" t="s">
         <v>156</v>
@@ -9480,8 +9480,8 @@
       <c r="G218">
         <v>76</v>
       </c>
-      <c r="H218">
-        <v>2</v>
+      <c r="H218" t="str">
+        <v>Europe</v>
       </c>
       <c r="I218" t="s">
         <v>26</v>
@@ -9517,8 +9517,8 @@
       <c r="G219">
         <v>76</v>
       </c>
-      <c r="H219">
-        <v>3</v>
+      <c r="H219" t="str">
+        <v>Asia</v>
       </c>
       <c r="I219" t="s">
         <v>111</v>
@@ -9554,8 +9554,8 @@
       <c r="G220">
         <v>76</v>
       </c>
-      <c r="H220">
-        <v>2</v>
+      <c r="H220" t="str">
+        <v>Europe</v>
       </c>
       <c r="I220" t="s">
         <v>157</v>
@@ -9591,8 +9591,8 @@
       <c r="G221">
         <v>76</v>
       </c>
-      <c r="H221">
-        <v>1</v>
+      <c r="H221" t="str">
+        <v>US</v>
       </c>
       <c r="I221" t="s">
         <v>158</v>
@@ -9628,8 +9628,8 @@
       <c r="G222">
         <v>76</v>
       </c>
-      <c r="H222">
-        <v>1</v>
+      <c r="H222" t="str">
+        <v>US</v>
       </c>
       <c r="I222" t="s">
         <v>159</v>
@@ -9665,8 +9665,8 @@
       <c r="G223">
         <v>76</v>
       </c>
-      <c r="H223">
-        <v>1</v>
+      <c r="H223" t="str">
+        <v>US</v>
       </c>
       <c r="I223" t="s">
         <v>160</v>
@@ -9702,8 +9702,8 @@
       <c r="G224">
         <v>76</v>
       </c>
-      <c r="H224">
-        <v>1</v>
+      <c r="H224" t="str">
+        <v>US</v>
       </c>
       <c r="I224" t="s">
         <v>161</v>
@@ -9739,8 +9739,8 @@
       <c r="G225">
         <v>77</v>
       </c>
-      <c r="H225">
-        <v>3</v>
+      <c r="H225" t="str">
+        <v>Asia</v>
       </c>
       <c r="I225" t="s">
         <v>162</v>
@@ -9776,8 +9776,8 @@
       <c r="G226">
         <v>77</v>
       </c>
-      <c r="H226">
-        <v>1</v>
+      <c r="H226" t="str">
+        <v>US</v>
       </c>
       <c r="I226" t="s">
         <v>163</v>
@@ -9813,8 +9813,8 @@
       <c r="G227">
         <v>77</v>
       </c>
-      <c r="H227">
-        <v>2</v>
+      <c r="H227" t="str">
+        <v>Europe</v>
       </c>
       <c r="I227" t="s">
         <v>164</v>
@@ -9850,8 +9850,8 @@
       <c r="G228">
         <v>77</v>
       </c>
-      <c r="H228">
-        <v>1</v>
+      <c r="H228" t="str">
+        <v>US</v>
       </c>
       <c r="I228" t="s">
         <v>165</v>
@@ -9887,8 +9887,8 @@
       <c r="G229">
         <v>77</v>
       </c>
-      <c r="H229">
-        <v>3</v>
+      <c r="H229" t="str">
+        <v>Asia</v>
       </c>
       <c r="I229" t="s">
         <v>166</v>
@@ -9924,8 +9924,8 @@
       <c r="G230">
         <v>77</v>
       </c>
-      <c r="H230">
-        <v>1</v>
+      <c r="H230" t="str">
+        <v>US</v>
       </c>
       <c r="I230" t="s">
         <v>86</v>
@@ -9961,8 +9961,8 @@
       <c r="G231">
         <v>77</v>
       </c>
-      <c r="H231">
-        <v>1</v>
+      <c r="H231" t="str">
+        <v>US</v>
       </c>
       <c r="I231" t="s">
         <v>167</v>
@@ -9998,8 +9998,8 @@
       <c r="G232">
         <v>77</v>
       </c>
-      <c r="H232">
-        <v>1</v>
+      <c r="H232" t="str">
+        <v>US</v>
       </c>
       <c r="I232" t="s">
         <v>168</v>
@@ -10035,8 +10035,8 @@
       <c r="G233">
         <v>77</v>
       </c>
-      <c r="H233">
-        <v>1</v>
+      <c r="H233" t="str">
+        <v>US</v>
       </c>
       <c r="I233" t="s">
         <v>169</v>
@@ -10072,8 +10072,8 @@
       <c r="G234">
         <v>77</v>
       </c>
-      <c r="H234">
-        <v>1</v>
+      <c r="H234" t="str">
+        <v>US</v>
       </c>
       <c r="I234" t="s">
         <v>170</v>
@@ -10109,8 +10109,8 @@
       <c r="G235">
         <v>77</v>
       </c>
-      <c r="H235">
-        <v>1</v>
+      <c r="H235" t="str">
+        <v>US</v>
       </c>
       <c r="I235" t="s">
         <v>171</v>
@@ -10146,8 +10146,8 @@
       <c r="G236">
         <v>77</v>
       </c>
-      <c r="H236">
-        <v>1</v>
+      <c r="H236" t="str">
+        <v>US</v>
       </c>
       <c r="I236" t="s">
         <v>172</v>
@@ -10183,8 +10183,8 @@
       <c r="G237">
         <v>77</v>
       </c>
-      <c r="H237">
-        <v>1</v>
+      <c r="H237" t="str">
+        <v>US</v>
       </c>
       <c r="I237" t="s">
         <v>173</v>
@@ -10220,8 +10220,8 @@
       <c r="G238">
         <v>77</v>
       </c>
-      <c r="H238">
-        <v>1</v>
+      <c r="H238" t="str">
+        <v>US</v>
       </c>
       <c r="I238" t="s">
         <v>174</v>
@@ -10257,8 +10257,8 @@
       <c r="G239">
         <v>77</v>
       </c>
-      <c r="H239">
-        <v>1</v>
+      <c r="H239" t="str">
+        <v>US</v>
       </c>
       <c r="I239" t="s">
         <v>175</v>
@@ -10294,8 +10294,8 @@
       <c r="G240">
         <v>77</v>
       </c>
-      <c r="H240">
-        <v>1</v>
+      <c r="H240" t="str">
+        <v>US</v>
       </c>
       <c r="I240" t="s">
         <v>176</v>
@@ -10331,8 +10331,8 @@
       <c r="G241">
         <v>77</v>
       </c>
-      <c r="H241">
-        <v>1</v>
+      <c r="H241" t="str">
+        <v>US</v>
       </c>
       <c r="I241" t="s">
         <v>177</v>
@@ -10368,8 +10368,8 @@
       <c r="G242">
         <v>77</v>
       </c>
-      <c r="H242">
-        <v>2</v>
+      <c r="H242" t="str">
+        <v>Europe</v>
       </c>
       <c r="I242" t="s">
         <v>178</v>
@@ -10405,8 +10405,8 @@
       <c r="G243">
         <v>77</v>
       </c>
-      <c r="H243">
-        <v>1</v>
+      <c r="H243" t="str">
+        <v>US</v>
       </c>
       <c r="I243" t="s">
         <v>179</v>
@@ -10442,8 +10442,8 @@
       <c r="G244">
         <v>77</v>
       </c>
-      <c r="H244">
-        <v>3</v>
+      <c r="H244" t="str">
+        <v>Asia</v>
       </c>
       <c r="I244" t="s">
         <v>180</v>
@@ -10479,8 +10479,8 @@
       <c r="G245">
         <v>77</v>
       </c>
-      <c r="H245">
-        <v>1</v>
+      <c r="H245" t="str">
+        <v>US</v>
       </c>
       <c r="I245" t="s">
         <v>181</v>
@@ -10516,8 +10516,8 @@
       <c r="G246">
         <v>77</v>
       </c>
-      <c r="H246">
-        <v>1</v>
+      <c r="H246" t="str">
+        <v>US</v>
       </c>
       <c r="I246" t="s">
         <v>147</v>
@@ -10553,8 +10553,8 @@
       <c r="G247">
         <v>77</v>
       </c>
-      <c r="H247">
-        <v>1</v>
+      <c r="H247" t="str">
+        <v>US</v>
       </c>
       <c r="I247" t="s">
         <v>182</v>
@@ -10590,8 +10590,8 @@
       <c r="G248">
         <v>77</v>
       </c>
-      <c r="H248">
-        <v>3</v>
+      <c r="H248" t="str">
+        <v>Asia</v>
       </c>
       <c r="I248" t="s">
         <v>183</v>
@@ -10627,8 +10627,8 @@
       <c r="G249">
         <v>77</v>
       </c>
-      <c r="H249">
-        <v>2</v>
+      <c r="H249" t="str">
+        <v>Europe</v>
       </c>
       <c r="I249" t="s">
         <v>120</v>
@@ -10664,8 +10664,8 @@
       <c r="G250">
         <v>77</v>
       </c>
-      <c r="H250">
-        <v>3</v>
+      <c r="H250" t="str">
+        <v>Asia</v>
       </c>
       <c r="I250" t="s">
         <v>184</v>
@@ -10701,8 +10701,8 @@
       <c r="G251">
         <v>77</v>
       </c>
-      <c r="H251">
-        <v>2</v>
+      <c r="H251" t="str">
+        <v>Europe</v>
       </c>
       <c r="I251" t="s">
         <v>185</v>
@@ -10738,8 +10738,8 @@
       <c r="G252">
         <v>77</v>
       </c>
-      <c r="H252">
-        <v>3</v>
+      <c r="H252" t="str">
+        <v>Asia</v>
       </c>
       <c r="I252" t="s">
         <v>186</v>
@@ -10775,8 +10775,8 @@
       <c r="G253">
         <v>78</v>
       </c>
-      <c r="H253">
-        <v>2</v>
+      <c r="H253" t="str">
+        <v>Europe</v>
       </c>
       <c r="I253" t="s">
         <v>187</v>
@@ -10812,8 +10812,8 @@
       <c r="G254">
         <v>78</v>
       </c>
-      <c r="H254">
-        <v>1</v>
+      <c r="H254" t="str">
+        <v>US</v>
       </c>
       <c r="I254" t="s">
         <v>188</v>
@@ -10849,8 +10849,8 @@
       <c r="G255">
         <v>78</v>
       </c>
-      <c r="H255">
-        <v>3</v>
+      <c r="H255" t="str">
+        <v>Asia</v>
       </c>
       <c r="I255" t="s">
         <v>189</v>
@@ -10886,8 +10886,8 @@
       <c r="G256">
         <v>78</v>
       </c>
-      <c r="H256">
-        <v>3</v>
+      <c r="H256" t="str">
+        <v>Asia</v>
       </c>
       <c r="I256" t="s">
         <v>190</v>
@@ -10923,8 +10923,8 @@
       <c r="G257">
         <v>78</v>
       </c>
-      <c r="H257">
-        <v>3</v>
+      <c r="H257" t="str">
+        <v>Asia</v>
       </c>
       <c r="I257" t="s">
         <v>142</v>
@@ -10960,8 +10960,8 @@
       <c r="G258">
         <v>78</v>
       </c>
-      <c r="H258">
-        <v>1</v>
+      <c r="H258" t="str">
+        <v>US</v>
       </c>
       <c r="I258" t="s">
         <v>191</v>
@@ -10997,8 +10997,8 @@
       <c r="G259">
         <v>78</v>
       </c>
-      <c r="H259">
-        <v>1</v>
+      <c r="H259" t="str">
+        <v>US</v>
       </c>
       <c r="I259" t="s">
         <v>192</v>
@@ -11034,8 +11034,8 @@
       <c r="G260">
         <v>78</v>
       </c>
-      <c r="H260">
-        <v>1</v>
+      <c r="H260" t="str">
+        <v>US</v>
       </c>
       <c r="I260" t="s">
         <v>193</v>
@@ -11071,8 +11071,8 @@
       <c r="G261">
         <v>78</v>
       </c>
-      <c r="H261">
-        <v>1</v>
+      <c r="H261" t="str">
+        <v>US</v>
       </c>
       <c r="I261" t="s">
         <v>194</v>
@@ -11108,8 +11108,8 @@
       <c r="G262">
         <v>78</v>
       </c>
-      <c r="H262">
-        <v>1</v>
+      <c r="H262" t="str">
+        <v>US</v>
       </c>
       <c r="I262" t="s">
         <v>82</v>
@@ -11145,8 +11145,8 @@
       <c r="G263">
         <v>78</v>
       </c>
-      <c r="H263">
-        <v>1</v>
+      <c r="H263" t="str">
+        <v>US</v>
       </c>
       <c r="I263" t="s">
         <v>195</v>
@@ -11182,8 +11182,8 @@
       <c r="G264">
         <v>78</v>
       </c>
-      <c r="H264">
-        <v>1</v>
+      <c r="H264" t="str">
+        <v>US</v>
       </c>
       <c r="I264" t="s">
         <v>196</v>
@@ -11219,8 +11219,8 @@
       <c r="G265">
         <v>78</v>
       </c>
-      <c r="H265">
-        <v>1</v>
+      <c r="H265" t="str">
+        <v>US</v>
       </c>
       <c r="I265" t="s">
         <v>197</v>
@@ -11256,8 +11256,8 @@
       <c r="G266">
         <v>78</v>
       </c>
-      <c r="H266">
-        <v>1</v>
+      <c r="H266" t="str">
+        <v>US</v>
       </c>
       <c r="I266" t="s">
         <v>198</v>
@@ -11293,8 +11293,8 @@
       <c r="G267">
         <v>78</v>
       </c>
-      <c r="H267">
-        <v>1</v>
+      <c r="H267" t="str">
+        <v>US</v>
       </c>
       <c r="I267" t="s">
         <v>199</v>
@@ -11330,8 +11330,8 @@
       <c r="G268">
         <v>78</v>
       </c>
-      <c r="H268">
-        <v>1</v>
+      <c r="H268" t="str">
+        <v>US</v>
       </c>
       <c r="I268" t="s">
         <v>200</v>
@@ -11367,8 +11367,8 @@
       <c r="G269">
         <v>78</v>
       </c>
-      <c r="H269">
-        <v>1</v>
+      <c r="H269" t="str">
+        <v>US</v>
       </c>
       <c r="I269" t="s">
         <v>201</v>
@@ -11404,8 +11404,8 @@
       <c r="G270">
         <v>78</v>
       </c>
-      <c r="H270">
-        <v>1</v>
+      <c r="H270" t="str">
+        <v>US</v>
       </c>
       <c r="I270" t="s">
         <v>202</v>
@@ -11441,8 +11441,8 @@
       <c r="G271">
         <v>78</v>
       </c>
-      <c r="H271">
-        <v>1</v>
+      <c r="H271" t="str">
+        <v>US</v>
       </c>
       <c r="I271" t="s">
         <v>175</v>
@@ -11478,8 +11478,8 @@
       <c r="G272">
         <v>78</v>
       </c>
-      <c r="H272">
-        <v>1</v>
+      <c r="H272" t="str">
+        <v>US</v>
       </c>
       <c r="I272" t="s">
         <v>203</v>
@@ -11515,8 +11515,8 @@
       <c r="G273">
         <v>78</v>
       </c>
-      <c r="H273">
-        <v>1</v>
+      <c r="H273" t="str">
+        <v>US</v>
       </c>
       <c r="I273" t="s">
         <v>204</v>
@@ -11552,8 +11552,8 @@
       <c r="G274">
         <v>78</v>
       </c>
-      <c r="H274">
-        <v>1</v>
+      <c r="H274" t="str">
+        <v>US</v>
       </c>
       <c r="I274" t="s">
         <v>205</v>
@@ -11589,8 +11589,8 @@
       <c r="G275">
         <v>78</v>
       </c>
-      <c r="H275">
-        <v>1</v>
+      <c r="H275" t="str">
+        <v>US</v>
       </c>
       <c r="I275" t="s">
         <v>147</v>
@@ -11626,8 +11626,8 @@
       <c r="G276">
         <v>78</v>
       </c>
-      <c r="H276">
-        <v>3</v>
+      <c r="H276" t="str">
+        <v>Asia</v>
       </c>
       <c r="I276" t="s">
         <v>36</v>
@@ -11663,8 +11663,8 @@
       <c r="G277">
         <v>78</v>
       </c>
-      <c r="H277">
-        <v>3</v>
+      <c r="H277" t="str">
+        <v>Asia</v>
       </c>
       <c r="I277" t="s">
         <v>206</v>
@@ -11700,8 +11700,8 @@
       <c r="G278">
         <v>78</v>
       </c>
-      <c r="H278">
-        <v>1</v>
+      <c r="H278" t="str">
+        <v>US</v>
       </c>
       <c r="I278" t="s">
         <v>207</v>
@@ -11737,8 +11737,8 @@
       <c r="G279">
         <v>78</v>
       </c>
-      <c r="H279">
-        <v>3</v>
+      <c r="H279" t="str">
+        <v>Asia</v>
       </c>
       <c r="I279" t="s">
         <v>208</v>
@@ -11774,8 +11774,8 @@
       <c r="G280">
         <v>78</v>
       </c>
-      <c r="H280">
-        <v>1</v>
+      <c r="H280" t="str">
+        <v>US</v>
       </c>
       <c r="I280" t="s">
         <v>209</v>
@@ -11811,8 +11811,8 @@
       <c r="G281">
         <v>78</v>
       </c>
-      <c r="H281">
-        <v>1</v>
+      <c r="H281" t="str">
+        <v>US</v>
       </c>
       <c r="I281" t="s">
         <v>210</v>
@@ -11848,8 +11848,8 @@
       <c r="G282">
         <v>78</v>
       </c>
-      <c r="H282">
-        <v>3</v>
+      <c r="H282" t="str">
+        <v>Asia</v>
       </c>
       <c r="I282" t="s">
         <v>211</v>
@@ -11885,8 +11885,8 @@
       <c r="G283">
         <v>78</v>
       </c>
-      <c r="H283">
-        <v>2</v>
+      <c r="H283" t="str">
+        <v>Europe</v>
       </c>
       <c r="I283" t="s">
         <v>212</v>
@@ -11922,8 +11922,8 @@
       <c r="G284">
         <v>78</v>
       </c>
-      <c r="H284">
-        <v>2</v>
+      <c r="H284" t="str">
+        <v>Europe</v>
       </c>
       <c r="I284" t="s">
         <v>213</v>
@@ -11959,8 +11959,8 @@
       <c r="G285">
         <v>78</v>
       </c>
-      <c r="H285">
-        <v>2</v>
+      <c r="H285" t="str">
+        <v>Europe</v>
       </c>
       <c r="I285" t="s">
         <v>214</v>
@@ -11996,8 +11996,8 @@
       <c r="G286">
         <v>78</v>
       </c>
-      <c r="H286">
-        <v>2</v>
+      <c r="H286" t="str">
+        <v>Europe</v>
       </c>
       <c r="I286" t="s">
         <v>215</v>
@@ -12033,8 +12033,8 @@
       <c r="G287">
         <v>78</v>
       </c>
-      <c r="H287">
-        <v>2</v>
+      <c r="H287" t="str">
+        <v>Europe</v>
       </c>
       <c r="I287" t="s">
         <v>216</v>
@@ -12070,8 +12070,8 @@
       <c r="G288">
         <v>78</v>
       </c>
-      <c r="H288">
-        <v>3</v>
+      <c r="H288" t="str">
+        <v>Asia</v>
       </c>
       <c r="I288" t="s">
         <v>217</v>
@@ -12107,8 +12107,8 @@
       <c r="G289">
         <v>79</v>
       </c>
-      <c r="H289">
-        <v>1</v>
+      <c r="H289" t="str">
+        <v>US</v>
       </c>
       <c r="I289" t="s">
         <v>218</v>
@@ -12144,8 +12144,8 @@
       <c r="G290">
         <v>79</v>
       </c>
-      <c r="H290">
-        <v>1</v>
+      <c r="H290" t="str">
+        <v>US</v>
       </c>
       <c r="I290" t="s">
         <v>219</v>
@@ -12181,8 +12181,8 @@
       <c r="G291">
         <v>79</v>
       </c>
-      <c r="H291">
-        <v>1</v>
+      <c r="H291" t="str">
+        <v>US</v>
       </c>
       <c r="I291" t="s">
         <v>220</v>
@@ -12218,8 +12218,8 @@
       <c r="G292">
         <v>79</v>
       </c>
-      <c r="H292">
-        <v>1</v>
+      <c r="H292" t="str">
+        <v>US</v>
       </c>
       <c r="I292" t="s">
         <v>221</v>
@@ -12255,8 +12255,8 @@
       <c r="G293">
         <v>79</v>
       </c>
-      <c r="H293">
-        <v>1</v>
+      <c r="H293" t="str">
+        <v>US</v>
       </c>
       <c r="I293" t="s">
         <v>222</v>
@@ -12292,8 +12292,8 @@
       <c r="G294">
         <v>79</v>
       </c>
-      <c r="H294">
-        <v>1</v>
+      <c r="H294" t="str">
+        <v>US</v>
       </c>
       <c r="I294" t="s">
         <v>86</v>
@@ -12329,8 +12329,8 @@
       <c r="G295">
         <v>79</v>
       </c>
-      <c r="H295">
-        <v>1</v>
+      <c r="H295" t="str">
+        <v>US</v>
       </c>
       <c r="I295" t="s">
         <v>223</v>
@@ -12366,8 +12366,8 @@
       <c r="G296">
         <v>79</v>
       </c>
-      <c r="H296">
-        <v>1</v>
+      <c r="H296" t="str">
+        <v>US</v>
       </c>
       <c r="I296" t="s">
         <v>224</v>
@@ -12403,8 +12403,8 @@
       <c r="G297">
         <v>79</v>
       </c>
-      <c r="H297">
-        <v>1</v>
+      <c r="H297" t="str">
+        <v>US</v>
       </c>
       <c r="I297" t="s">
         <v>225</v>
@@ -12440,8 +12440,8 @@
       <c r="G298">
         <v>79</v>
       </c>
-      <c r="H298">
-        <v>1</v>
+      <c r="H298" t="str">
+        <v>US</v>
       </c>
       <c r="I298" t="s">
         <v>19</v>
@@ -12477,8 +12477,8 @@
       <c r="G299">
         <v>79</v>
       </c>
-      <c r="H299">
-        <v>1</v>
+      <c r="H299" t="str">
+        <v>US</v>
       </c>
       <c r="I299" t="s">
         <v>44</v>
@@ -12514,8 +12514,8 @@
       <c r="G300">
         <v>79</v>
       </c>
-      <c r="H300">
-        <v>1</v>
+      <c r="H300" t="str">
+        <v>US</v>
       </c>
       <c r="I300" t="s">
         <v>226</v>
@@ -12551,8 +12551,8 @@
       <c r="G301">
         <v>79</v>
       </c>
-      <c r="H301">
-        <v>1</v>
+      <c r="H301" t="str">
+        <v>US</v>
       </c>
       <c r="I301" t="s">
         <v>227</v>
@@ -12588,8 +12588,8 @@
       <c r="G302">
         <v>79</v>
       </c>
-      <c r="H302">
-        <v>2</v>
+      <c r="H302" t="str">
+        <v>Europe</v>
       </c>
       <c r="I302" t="s">
         <v>228</v>
@@ -12625,8 +12625,8 @@
       <c r="G303">
         <v>79</v>
       </c>
-      <c r="H303">
-        <v>3</v>
+      <c r="H303" t="str">
+        <v>Asia</v>
       </c>
       <c r="I303" t="s">
         <v>229</v>
@@ -12662,8 +12662,8 @@
       <c r="G304">
         <v>79</v>
       </c>
-      <c r="H304">
-        <v>1</v>
+      <c r="H304" t="str">
+        <v>US</v>
       </c>
       <c r="I304" t="s">
         <v>230</v>
@@ -12699,8 +12699,8 @@
       <c r="G305">
         <v>79</v>
       </c>
-      <c r="H305">
-        <v>1</v>
+      <c r="H305" t="str">
+        <v>US</v>
       </c>
       <c r="I305" t="s">
         <v>231</v>
@@ -12736,8 +12736,8 @@
       <c r="G306">
         <v>79</v>
       </c>
-      <c r="H306">
-        <v>2</v>
+      <c r="H306" t="str">
+        <v>Europe</v>
       </c>
       <c r="I306" t="s">
         <v>232</v>
@@ -12773,8 +12773,8 @@
       <c r="G307">
         <v>79</v>
       </c>
-      <c r="H307">
-        <v>1</v>
+      <c r="H307" t="str">
+        <v>US</v>
       </c>
       <c r="I307" t="s">
         <v>233</v>
@@ -12810,8 +12810,8 @@
       <c r="G308">
         <v>79</v>
       </c>
-      <c r="H308">
-        <v>2</v>
+      <c r="H308" t="str">
+        <v>Europe</v>
       </c>
       <c r="I308" t="s">
         <v>26</v>
@@ -12847,8 +12847,8 @@
       <c r="G309">
         <v>79</v>
       </c>
-      <c r="H309">
-        <v>1</v>
+      <c r="H309" t="str">
+        <v>US</v>
       </c>
       <c r="I309" t="s">
         <v>191</v>
@@ -12884,8 +12884,8 @@
       <c r="G310">
         <v>79</v>
       </c>
-      <c r="H310">
-        <v>1</v>
+      <c r="H310" t="str">
+        <v>US</v>
       </c>
       <c r="I310" t="s">
         <v>234</v>
@@ -12921,8 +12921,8 @@
       <c r="G311">
         <v>79</v>
       </c>
-      <c r="H311">
-        <v>1</v>
+      <c r="H311" t="str">
+        <v>US</v>
       </c>
       <c r="I311" t="s">
         <v>235</v>
@@ -12958,8 +12958,8 @@
       <c r="G312">
         <v>79</v>
       </c>
-      <c r="H312">
-        <v>3</v>
+      <c r="H312" t="str">
+        <v>Asia</v>
       </c>
       <c r="I312" t="s">
         <v>236</v>
@@ -12995,8 +12995,8 @@
       <c r="G313">
         <v>79</v>
       </c>
-      <c r="H313">
-        <v>2</v>
+      <c r="H313" t="str">
+        <v>Europe</v>
       </c>
       <c r="I313" t="s">
         <v>237</v>
@@ -13032,8 +13032,8 @@
       <c r="G314">
         <v>79</v>
       </c>
-      <c r="H314">
-        <v>1</v>
+      <c r="H314" t="str">
+        <v>US</v>
       </c>
       <c r="I314" t="s">
         <v>238</v>
@@ -13069,8 +13069,8 @@
       <c r="G315">
         <v>79</v>
       </c>
-      <c r="H315">
-        <v>1</v>
+      <c r="H315" t="str">
+        <v>US</v>
       </c>
       <c r="I315" t="s">
         <v>239</v>
@@ -13106,8 +13106,8 @@
       <c r="G316">
         <v>79</v>
       </c>
-      <c r="H316">
-        <v>1</v>
+      <c r="H316" t="str">
+        <v>US</v>
       </c>
       <c r="I316" t="s">
         <v>240</v>
@@ -13143,8 +13143,8 @@
       <c r="G317">
         <v>79</v>
       </c>
-      <c r="H317">
-        <v>1</v>
+      <c r="H317" t="str">
+        <v>US</v>
       </c>
       <c r="I317" t="s">
         <v>241</v>
@@ -13180,8 +13180,8 @@
       <c r="G318">
         <v>80</v>
       </c>
-      <c r="H318">
-        <v>2</v>
+      <c r="H318" t="str">
+        <v>Europe</v>
       </c>
       <c r="I318" t="s">
         <v>149</v>
@@ -13217,8 +13217,8 @@
       <c r="G319">
         <v>80</v>
       </c>
-      <c r="H319">
-        <v>3</v>
+      <c r="H319" t="str">
+        <v>Asia</v>
       </c>
       <c r="I319" t="s">
         <v>242</v>
@@ -13254,8 +13254,8 @@
       <c r="G320">
         <v>80</v>
       </c>
-      <c r="H320">
-        <v>1</v>
+      <c r="H320" t="str">
+        <v>US</v>
       </c>
       <c r="I320" t="s">
         <v>147</v>
@@ -13291,8 +13291,8 @@
       <c r="G321">
         <v>80</v>
       </c>
-      <c r="H321">
-        <v>3</v>
+      <c r="H321" t="str">
+        <v>Asia</v>
       </c>
       <c r="I321" t="s">
         <v>243</v>
@@ -13328,8 +13328,8 @@
       <c r="G322">
         <v>80</v>
       </c>
-      <c r="H322">
-        <v>1</v>
+      <c r="H322" t="str">
+        <v>US</v>
       </c>
       <c r="I322" t="s">
         <v>239</v>
@@ -13365,8 +13365,8 @@
       <c r="G323">
         <v>80</v>
       </c>
-      <c r="H323">
-        <v>1</v>
+      <c r="H323" t="str">
+        <v>US</v>
       </c>
       <c r="I323" t="s">
         <v>244</v>
@@ -13402,8 +13402,8 @@
       <c r="G324">
         <v>80</v>
       </c>
-      <c r="H324">
-        <v>1</v>
+      <c r="H324" t="str">
+        <v>US</v>
       </c>
       <c r="I324" t="s">
         <v>198</v>
@@ -13439,8 +13439,8 @@
       <c r="G325">
         <v>80</v>
       </c>
-      <c r="H325">
-        <v>1</v>
+      <c r="H325" t="str">
+        <v>US</v>
       </c>
       <c r="I325" t="s">
         <v>201</v>
@@ -13476,8 +13476,8 @@
       <c r="G326">
         <v>80</v>
       </c>
-      <c r="H326">
-        <v>2</v>
+      <c r="H326" t="str">
+        <v>Europe</v>
       </c>
       <c r="I326" t="s">
         <v>245</v>
@@ -13513,8 +13513,8 @@
       <c r="G327">
         <v>80</v>
       </c>
-      <c r="H327">
-        <v>3</v>
+      <c r="H327" t="str">
+        <v>Asia</v>
       </c>
       <c r="I327" t="s">
         <v>246</v>
@@ -13550,8 +13550,8 @@
       <c r="G328">
         <v>80</v>
       </c>
-      <c r="H328">
-        <v>3</v>
+      <c r="H328" t="str">
+        <v>Asia</v>
       </c>
       <c r="I328" t="s">
         <v>247</v>
@@ -13587,8 +13587,8 @@
       <c r="G329">
         <v>80</v>
       </c>
-      <c r="H329">
-        <v>3</v>
+      <c r="H329" t="str">
+        <v>Asia</v>
       </c>
       <c r="I329" t="s">
         <v>248</v>
@@ -13624,8 +13624,8 @@
       <c r="G330">
         <v>80</v>
       </c>
-      <c r="H330">
-        <v>3</v>
+      <c r="H330" t="str">
+        <v>Asia</v>
       </c>
       <c r="I330" t="s">
         <v>137</v>
@@ -13661,8 +13661,8 @@
       <c r="G331">
         <v>80</v>
       </c>
-      <c r="H331">
-        <v>3</v>
+      <c r="H331" t="str">
+        <v>Asia</v>
       </c>
       <c r="I331" t="s">
         <v>249</v>
@@ -13698,8 +13698,8 @@
       <c r="G332">
         <v>80</v>
       </c>
-      <c r="H332">
-        <v>1</v>
+      <c r="H332" t="str">
+        <v>US</v>
       </c>
       <c r="I332" t="s">
         <v>122</v>
@@ -13735,8 +13735,8 @@
       <c r="G333">
         <v>80</v>
       </c>
-      <c r="H333">
-        <v>3</v>
+      <c r="H333" t="str">
+        <v>Asia</v>
       </c>
       <c r="I333" t="s">
         <v>236</v>
@@ -13772,8 +13772,8 @@
       <c r="G334">
         <v>80</v>
       </c>
-      <c r="H334">
-        <v>2</v>
+      <c r="H334" t="str">
+        <v>Europe</v>
       </c>
       <c r="I334" t="s">
         <v>250</v>
@@ -13809,8 +13809,8 @@
       <c r="G335">
         <v>80</v>
       </c>
-      <c r="H335">
-        <v>2</v>
+      <c r="H335" t="str">
+        <v>Europe</v>
       </c>
       <c r="I335" t="s">
         <v>251</v>
@@ -13846,8 +13846,8 @@
       <c r="G336">
         <v>80</v>
       </c>
-      <c r="H336">
-        <v>2</v>
+      <c r="H336" t="str">
+        <v>Europe</v>
       </c>
       <c r="I336" t="s">
         <v>252</v>
@@ -13883,8 +13883,8 @@
       <c r="G337">
         <v>80</v>
       </c>
-      <c r="H337">
-        <v>2</v>
+      <c r="H337" t="str">
+        <v>Europe</v>
       </c>
       <c r="I337" t="s">
         <v>253</v>
@@ -13920,8 +13920,8 @@
       <c r="G338">
         <v>80</v>
       </c>
-      <c r="H338">
-        <v>3</v>
+      <c r="H338" t="str">
+        <v>Asia</v>
       </c>
       <c r="I338" t="s">
         <v>254</v>
@@ -13957,8 +13957,8 @@
       <c r="G339">
         <v>80</v>
       </c>
-      <c r="H339">
-        <v>2</v>
+      <c r="H339" t="str">
+        <v>Europe</v>
       </c>
       <c r="I339" t="s">
         <v>255</v>
@@ -13994,8 +13994,8 @@
       <c r="G340">
         <v>80</v>
       </c>
-      <c r="H340">
-        <v>3</v>
+      <c r="H340" t="str">
+        <v>Asia</v>
       </c>
       <c r="I340" t="s">
         <v>183</v>
@@ -14031,8 +14031,8 @@
       <c r="G341">
         <v>80</v>
       </c>
-      <c r="H341">
-        <v>2</v>
+      <c r="H341" t="str">
+        <v>Europe</v>
       </c>
       <c r="I341" t="s">
         <v>256</v>
@@ -14068,8 +14068,8 @@
       <c r="G342">
         <v>80</v>
       </c>
-      <c r="H342">
-        <v>3</v>
+      <c r="H342" t="str">
+        <v>Asia</v>
       </c>
       <c r="I342" t="s">
         <v>257</v>
@@ -14105,8 +14105,8 @@
       <c r="G343">
         <v>80</v>
       </c>
-      <c r="H343">
-        <v>3</v>
+      <c r="H343" t="str">
+        <v>Asia</v>
       </c>
       <c r="I343" t="s">
         <v>258</v>
@@ -14142,8 +14142,8 @@
       <c r="G344">
         <v>80</v>
       </c>
-      <c r="H344">
-        <v>2</v>
+      <c r="H344" t="str">
+        <v>Europe</v>
       </c>
       <c r="I344" t="s">
         <v>259</v>
@@ -14179,8 +14179,8 @@
       <c r="G345">
         <v>80</v>
       </c>
-      <c r="H345">
-        <v>1</v>
+      <c r="H345" t="str">
+        <v>US</v>
       </c>
       <c r="I345" t="s">
         <v>260</v>
@@ -14216,8 +14216,8 @@
       <c r="G346">
         <v>80</v>
       </c>
-      <c r="H346">
-        <v>3</v>
+      <c r="H346" t="str">
+        <v>Asia</v>
       </c>
       <c r="I346" t="s">
         <v>261</v>
@@ -14253,8 +14253,8 @@
       <c r="G347">
         <v>81</v>
       </c>
-      <c r="H347">
-        <v>1</v>
+      <c r="H347" t="str">
+        <v>US</v>
       </c>
       <c r="I347" t="s">
         <v>262</v>
@@ -14290,8 +14290,8 @@
       <c r="G348">
         <v>81</v>
       </c>
-      <c r="H348">
-        <v>1</v>
+      <c r="H348" t="str">
+        <v>US</v>
       </c>
       <c r="I348" t="s">
         <v>171</v>
@@ -14327,8 +14327,8 @@
       <c r="G349">
         <v>81</v>
       </c>
-      <c r="H349">
-        <v>1</v>
+      <c r="H349" t="str">
+        <v>US</v>
       </c>
       <c r="I349" t="s">
         <v>263</v>
@@ -14364,8 +14364,8 @@
       <c r="G350">
         <v>81</v>
       </c>
-      <c r="H350">
-        <v>1</v>
+      <c r="H350" t="str">
+        <v>US</v>
       </c>
       <c r="I350" t="s">
         <v>239</v>
@@ -14401,8 +14401,8 @@
       <c r="G351">
         <v>81</v>
       </c>
-      <c r="H351">
-        <v>1</v>
+      <c r="H351" t="str">
+        <v>US</v>
       </c>
       <c r="I351" t="s">
         <v>262</v>
@@ -14438,8 +14438,8 @@
       <c r="G352">
         <v>81</v>
       </c>
-      <c r="H352">
-        <v>3</v>
+      <c r="H352" t="str">
+        <v>Asia</v>
       </c>
       <c r="I352" t="s">
         <v>264</v>
@@ -14475,8 +14475,8 @@
       <c r="G353">
         <v>81</v>
       </c>
-      <c r="H353">
-        <v>1</v>
+      <c r="H353" t="str">
+        <v>US</v>
       </c>
       <c r="I353" t="s">
         <v>265</v>
@@ -14512,8 +14512,8 @@
       <c r="G354">
         <v>81</v>
       </c>
-      <c r="H354">
-        <v>3</v>
+      <c r="H354" t="str">
+        <v>Asia</v>
       </c>
       <c r="I354" t="s">
         <v>266</v>
@@ -14549,8 +14549,8 @@
       <c r="G355">
         <v>81</v>
       </c>
-      <c r="H355">
-        <v>3</v>
+      <c r="H355" t="str">
+        <v>Asia</v>
       </c>
       <c r="I355" t="s">
         <v>125</v>
@@ -14586,8 +14586,8 @@
       <c r="G356">
         <v>81</v>
       </c>
-      <c r="H356">
-        <v>3</v>
+      <c r="H356" t="str">
+        <v>Asia</v>
       </c>
       <c r="I356" t="s">
         <v>267</v>
@@ -14623,8 +14623,8 @@
       <c r="G357">
         <v>81</v>
       </c>
-      <c r="H357">
-        <v>3</v>
+      <c r="H357" t="str">
+        <v>Asia</v>
       </c>
       <c r="I357" t="s">
         <v>268</v>
@@ -14660,8 +14660,8 @@
       <c r="G358">
         <v>81</v>
       </c>
-      <c r="H358">
-        <v>3</v>
+      <c r="H358" t="str">
+        <v>Asia</v>
       </c>
       <c r="I358" t="s">
         <v>269</v>
@@ -14697,8 +14697,8 @@
       <c r="G359">
         <v>81</v>
       </c>
-      <c r="H359">
-        <v>1</v>
+      <c r="H359" t="str">
+        <v>US</v>
       </c>
       <c r="I359" t="s">
         <v>270</v>
@@ -14734,8 +14734,8 @@
       <c r="G360">
         <v>81</v>
       </c>
-      <c r="H360">
-        <v>1</v>
+      <c r="H360" t="str">
+        <v>US</v>
       </c>
       <c r="I360" t="s">
         <v>271</v>
@@ -14771,8 +14771,8 @@
       <c r="G361">
         <v>81</v>
       </c>
-      <c r="H361">
-        <v>1</v>
+      <c r="H361" t="str">
+        <v>US</v>
       </c>
       <c r="I361" t="s">
         <v>272</v>
@@ -14808,8 +14808,8 @@
       <c r="G362">
         <v>81</v>
       </c>
-      <c r="H362">
-        <v>2</v>
+      <c r="H362" t="str">
+        <v>Europe</v>
       </c>
       <c r="I362" t="s">
         <v>273</v>
@@ -14845,8 +14845,8 @@
       <c r="G363">
         <v>81</v>
       </c>
-      <c r="H363">
-        <v>2</v>
+      <c r="H363" t="str">
+        <v>Europe</v>
       </c>
       <c r="I363" t="s">
         <v>274</v>
@@ -14882,8 +14882,8 @@
       <c r="G364">
         <v>81</v>
       </c>
-      <c r="H364">
-        <v>3</v>
+      <c r="H364" t="str">
+        <v>Asia</v>
       </c>
       <c r="I364" t="s">
         <v>275</v>
@@ -14919,8 +14919,8 @@
       <c r="G365">
         <v>81</v>
       </c>
-      <c r="H365">
-        <v>3</v>
+      <c r="H365" t="str">
+        <v>Asia</v>
       </c>
       <c r="I365" t="s">
         <v>137</v>
@@ -14956,8 +14956,8 @@
       <c r="G366">
         <v>81</v>
       </c>
-      <c r="H366">
-        <v>3</v>
+      <c r="H366" t="str">
+        <v>Asia</v>
       </c>
       <c r="I366" t="s">
         <v>276</v>
@@ -14993,8 +14993,8 @@
       <c r="G367">
         <v>81</v>
       </c>
-      <c r="H367">
-        <v>3</v>
+      <c r="H367" t="str">
+        <v>Asia</v>
       </c>
       <c r="I367" t="s">
         <v>247</v>
@@ -15030,8 +15030,8 @@
       <c r="G368">
         <v>81</v>
       </c>
-      <c r="H368">
-        <v>2</v>
+      <c r="H368" t="str">
+        <v>Europe</v>
       </c>
       <c r="I368" t="s">
         <v>277</v>
@@ -15067,8 +15067,8 @@
       <c r="G369">
         <v>81</v>
       </c>
-      <c r="H369">
-        <v>2</v>
+      <c r="H369" t="str">
+        <v>Europe</v>
       </c>
       <c r="I369" t="s">
         <v>278</v>
@@ -15104,8 +15104,8 @@
       <c r="G370">
         <v>81</v>
       </c>
-      <c r="H370">
-        <v>2</v>
+      <c r="H370" t="str">
+        <v>Europe</v>
       </c>
       <c r="I370" t="s">
         <v>279</v>
@@ -15141,8 +15141,8 @@
       <c r="G371">
         <v>81</v>
       </c>
-      <c r="H371">
-        <v>3</v>
+      <c r="H371" t="str">
+        <v>Asia</v>
       </c>
       <c r="I371" t="s">
         <v>280</v>
@@ -15178,8 +15178,8 @@
       <c r="G372">
         <v>81</v>
       </c>
-      <c r="H372">
-        <v>3</v>
+      <c r="H372" t="str">
+        <v>Asia</v>
       </c>
       <c r="I372" t="s">
         <v>281</v>
@@ -15215,8 +15215,8 @@
       <c r="G373">
         <v>81</v>
       </c>
-      <c r="H373">
-        <v>1</v>
+      <c r="H373" t="str">
+        <v>US</v>
       </c>
       <c r="I373" t="s">
         <v>131</v>
@@ -15252,8 +15252,8 @@
       <c r="G374">
         <v>81</v>
       </c>
-      <c r="H374">
-        <v>1</v>
+      <c r="H374" t="str">
+        <v>US</v>
       </c>
       <c r="I374" t="s">
         <v>282</v>
@@ -15289,8 +15289,8 @@
       <c r="G375">
         <v>81</v>
       </c>
-      <c r="H375">
-        <v>1</v>
+      <c r="H375" t="str">
+        <v>US</v>
       </c>
       <c r="I375" t="s">
         <v>283</v>
@@ -15326,8 +15326,8 @@
       <c r="G376">
         <v>81</v>
       </c>
-      <c r="H376">
-        <v>1</v>
+      <c r="H376" t="str">
+        <v>US</v>
       </c>
       <c r="I376" t="s">
         <v>284</v>
@@ -15363,8 +15363,8 @@
       <c r="G377">
         <v>82</v>
       </c>
-      <c r="H377">
-        <v>1</v>
+      <c r="H377" t="str">
+        <v>US</v>
       </c>
       <c r="I377" t="s">
         <v>285</v>
@@ -15400,8 +15400,8 @@
       <c r="G378">
         <v>82</v>
       </c>
-      <c r="H378">
-        <v>1</v>
+      <c r="H378" t="str">
+        <v>US</v>
       </c>
       <c r="I378" t="s">
         <v>286</v>
@@ -15437,8 +15437,8 @@
       <c r="G379">
         <v>82</v>
       </c>
-      <c r="H379">
-        <v>1</v>
+      <c r="H379" t="str">
+        <v>US</v>
       </c>
       <c r="I379" t="s">
         <v>287</v>
@@ -15474,8 +15474,8 @@
       <c r="G380">
         <v>82</v>
       </c>
-      <c r="H380">
-        <v>1</v>
+      <c r="H380" t="str">
+        <v>US</v>
       </c>
       <c r="I380" t="s">
         <v>288</v>
@@ -15511,8 +15511,8 @@
       <c r="G381">
         <v>82</v>
       </c>
-      <c r="H381">
-        <v>1</v>
+      <c r="H381" t="str">
+        <v>US</v>
       </c>
       <c r="I381" t="s">
         <v>289</v>
@@ -15548,8 +15548,8 @@
       <c r="G382">
         <v>82</v>
       </c>
-      <c r="H382">
-        <v>1</v>
+      <c r="H382" t="str">
+        <v>US</v>
       </c>
       <c r="I382" t="s">
         <v>241</v>
@@ -15585,8 +15585,8 @@
       <c r="G383">
         <v>82</v>
       </c>
-      <c r="H383">
-        <v>1</v>
+      <c r="H383" t="str">
+        <v>US</v>
       </c>
       <c r="I383" t="s">
         <v>290</v>
@@ -15622,8 +15622,8 @@
       <c r="G384">
         <v>82</v>
       </c>
-      <c r="H384">
-        <v>1</v>
+      <c r="H384" t="str">
+        <v>US</v>
       </c>
       <c r="I384" t="s">
         <v>291</v>
@@ -15659,8 +15659,8 @@
       <c r="G385">
         <v>82</v>
       </c>
-      <c r="H385">
-        <v>2</v>
+      <c r="H385" t="str">
+        <v>Europe</v>
       </c>
       <c r="I385" t="s">
         <v>292</v>
@@ -15696,8 +15696,8 @@
       <c r="G386">
         <v>82</v>
       </c>
-      <c r="H386">
-        <v>3</v>
+      <c r="H386" t="str">
+        <v>Asia</v>
       </c>
       <c r="I386" t="s">
         <v>293</v>
@@ -15733,8 +15733,8 @@
       <c r="G387">
         <v>82</v>
       </c>
-      <c r="H387">
-        <v>3</v>
+      <c r="H387" t="str">
+        <v>Asia</v>
       </c>
       <c r="I387" t="s">
         <v>294</v>
@@ -15770,8 +15770,8 @@
       <c r="G388">
         <v>82</v>
       </c>
-      <c r="H388">
-        <v>1</v>
+      <c r="H388" t="str">
+        <v>US</v>
       </c>
       <c r="I388" t="s">
         <v>295</v>
@@ -15807,8 +15807,8 @@
       <c r="G389">
         <v>82</v>
       </c>
-      <c r="H389">
-        <v>1</v>
+      <c r="H389" t="str">
+        <v>US</v>
       </c>
       <c r="I389" t="s">
         <v>296</v>
@@ -15844,8 +15844,8 @@
       <c r="G390">
         <v>82</v>
       </c>
-      <c r="H390">
-        <v>3</v>
+      <c r="H390" t="str">
+        <v>Asia</v>
       </c>
       <c r="I390" t="s">
         <v>297</v>
@@ -15881,8 +15881,8 @@
       <c r="G391">
         <v>82</v>
       </c>
-      <c r="H391">
-        <v>3</v>
+      <c r="H391" t="str">
+        <v>Asia</v>
       </c>
       <c r="I391" t="s">
         <v>261</v>
@@ -15918,8 +15918,8 @@
       <c r="G392">
         <v>82</v>
       </c>
-      <c r="H392">
-        <v>3</v>
+      <c r="H392" t="str">
+        <v>Asia</v>
       </c>
       <c r="I392" t="s">
         <v>137</v>
@@ -15955,8 +15955,8 @@
       <c r="G393">
         <v>82</v>
       </c>
-      <c r="H393">
-        <v>3</v>
+      <c r="H393" t="str">
+        <v>Asia</v>
       </c>
       <c r="I393" t="s">
         <v>124</v>
@@ -15992,8 +15992,8 @@
       <c r="G394">
         <v>82</v>
       </c>
-      <c r="H394">
-        <v>3</v>
+      <c r="H394" t="str">
+        <v>Asia</v>
       </c>
       <c r="I394" t="s">
         <v>298</v>
@@ -16029,8 +16029,8 @@
       <c r="G395">
         <v>82</v>
       </c>
-      <c r="H395">
-        <v>3</v>
+      <c r="H395" t="str">
+        <v>Asia</v>
       </c>
       <c r="I395" t="s">
         <v>299</v>
@@ -16066,8 +16066,8 @@
       <c r="G396">
         <v>82</v>
       </c>
-      <c r="H396">
-        <v>1</v>
+      <c r="H396" t="str">
+        <v>US</v>
       </c>
       <c r="I396" t="s">
         <v>300</v>
@@ -16103,8 +16103,8 @@
       <c r="G397">
         <v>82</v>
       </c>
-      <c r="H397">
-        <v>1</v>
+      <c r="H397" t="str">
+        <v>US</v>
       </c>
       <c r="I397" t="s">
         <v>301</v>
@@ -16140,8 +16140,8 @@
       <c r="G398">
         <v>82</v>
       </c>
-      <c r="H398">
-        <v>1</v>
+      <c r="H398" t="str">
+        <v>US</v>
       </c>
       <c r="I398" t="s">
         <v>302</v>
@@ -16177,8 +16177,8 @@
       <c r="G399">
         <v>82</v>
       </c>
-      <c r="H399">
-        <v>1</v>
+      <c r="H399" t="str">
+        <v>US</v>
       </c>
       <c r="I399" t="s">
         <v>303</v>
@@ -16214,8 +16214,8 @@
       <c r="G400">
         <v>82</v>
       </c>
-      <c r="H400">
-        <v>3</v>
+      <c r="H400" t="str">
+        <v>Asia</v>
       </c>
       <c r="I400" t="s">
         <v>304</v>
@@ -16251,8 +16251,8 @@
       <c r="G401">
         <v>82</v>
       </c>
-      <c r="H401">
-        <v>1</v>
+      <c r="H401" t="str">
+        <v>US</v>
       </c>
       <c r="I401" t="s">
         <v>305</v>
@@ -16288,8 +16288,8 @@
       <c r="G402">
         <v>82</v>
       </c>
-      <c r="H402">
-        <v>1</v>
+      <c r="H402" t="str">
+        <v>US</v>
       </c>
       <c r="I402" t="s">
         <v>306</v>
@@ -16325,8 +16325,8 @@
       <c r="G403">
         <v>82</v>
       </c>
-      <c r="H403">
-        <v>1</v>
+      <c r="H403" t="str">
+        <v>US</v>
       </c>
       <c r="I403" t="s">
         <v>307</v>
@@ -16362,8 +16362,8 @@
       <c r="G404">
         <v>82</v>
       </c>
-      <c r="H404">
-        <v>2</v>
+      <c r="H404" t="str">
+        <v>Europe</v>
       </c>
       <c r="I404" t="s">
         <v>308</v>
@@ -16399,8 +16399,8 @@
       <c r="G405">
         <v>82</v>
       </c>
-      <c r="H405">
-        <v>1</v>
+      <c r="H405" t="str">
+        <v>US</v>
       </c>
       <c r="I405" t="s">
         <v>309</v>
@@ -16436,8 +16436,8 @@
       <c r="G406">
         <v>82</v>
       </c>
-      <c r="H406">
-        <v>1</v>
+      <c r="H406" t="str">
+        <v>US</v>
       </c>
       <c r="I406" t="s">
         <v>310</v>
@@ -16473,8 +16473,8 @@
       <c r="G407">
         <v>82</v>
       </c>
-      <c r="H407">
-        <v>1</v>
+      <c r="H407" t="str">
+        <v>US</v>
       </c>
       <c r="I407" t="s">
         <v>311</v>

</xml_diff>